<commit_message>
Weekly NBA competitor report 2026-09-13
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 06 September 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 13 September 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,425</t>
+          <t>18,529</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+1.24%</t>
+          <t>+1.81%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+225 followers • 54 days</t>
+          <t>+329 followers • 61 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>57539</v>
+        <v>57884</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -1272,14 +1272,14 @@
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.0571</v>
+        <v>0.0733</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>54d</t>
+          <t>61d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18425</v>
+        <v>18529</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
@@ -1306,14 +1306,14 @@
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.047</v>
+        <v>0.0605</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>54d</t>
+          <t>61d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,25 +1329,25 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>17835</v>
+        <v>17865</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>@icnnewzealand</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>217</v>
+        <v>63</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.0344</v>
+        <v>0.045</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>54d</t>
+          <t>61d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,25 +1363,25 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>16036</v>
+        <v>16135</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>@ifbbproleagueoz</t>
+          <t>@icnnewzealand</t>
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>1439</v>
+        <v>239</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0257</v>
+        <v>0.0379</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>54d</t>
+          <t>61d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,25 +1397,25 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15721</v>
+        <v>15715</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>@anb.australia</t>
+          <t>@wnbfaustralia</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.0246</v>
+        <v>0.0338</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>54d</t>
+          <t>61d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>57539</v>
+        <v>57884</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.0571</v>
+        <v>0.0733</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,7 +1826,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18425</v>
+        <v>18529</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.047</v>
+        <v>0.0605</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,15 +1844,15 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17835</v>
+        <v>17865</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>@icnnewzealand</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.0344</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,15 +1862,15 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16036</v>
+        <v>16135</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>@ifbbproleagueoz</t>
+          <t>@icnnewzealand</t>
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0257</v>
+        <v>0.0379</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,15 +1880,15 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15721</v>
+        <v>15715</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>@anb.australia</t>
+          <t>@wnbfaustralia</t>
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.0246</v>
+        <v>0.0338</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,13 +2002,13 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>57539</v>
+        <v>57884</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>1439</v>
+        <v>1784</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0257</v>
+        <v>0.0318</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
@@ -2016,13 +2016,13 @@
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H2" s="27" t="n">
-        <v>7970</v>
+        <v>8050</v>
       </c>
       <c r="I2" s="28" t="n">
-        <v>168</v>
+        <v>80</v>
       </c>
       <c r="J2" s="26" t="inlineStr">
         <is>
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18425</v>
+        <v>18529</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>225</v>
+        <v>329</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0124</v>
+        <v>0.0181</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
@@ -2054,13 +2054,13 @@
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3335</v>
+        <v>3355</v>
       </c>
       <c r="I3" s="28" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
@@ -2078,13 +2078,13 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>17835</v>
+        <v>17865</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0076</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2092,13 +2092,13 @@
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6786</v>
+        <v>6795</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2116,13 +2116,13 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>16036</v>
+        <v>16135</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>236</v>
+        <v>335</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0149</v>
+        <v>0.0212</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
@@ -2130,13 +2130,13 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>6786</v>
+        <v>6848</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
@@ -2154,13 +2154,13 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15721</v>
+        <v>15715</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>-179</v>
+        <v>-185</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>-0.0113</v>
+        <v>-0.0116</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -2168,13 +2168,13 @@
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>2970</v>
+        <v>2975</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
@@ -2192,13 +2192,13 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15466</v>
+        <v>15507</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>266</v>
+        <v>307</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0175</v>
+        <v>0.0202</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
@@ -2206,13 +2206,13 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3589</v>
+        <v>3596</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J7" s="26" t="inlineStr">
         <is>
@@ -2230,13 +2230,13 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>12893</v>
+        <v>12963</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>193</v>
+        <v>263</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0152</v>
+        <v>0.0207</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -2244,13 +2244,13 @@
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4462</v>
+        <v>4468</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
@@ -2268,13 +2268,13 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11413</v>
+        <v>11420</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.01</v>
+        <v>0.0106</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
@@ -2282,13 +2282,13 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2846</v>
+        <v>2852</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,13 +2306,13 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>10997</v>
+        <v>11018</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>-3</v>
-      </c>
-      <c r="E10" s="30" t="n">
-        <v>-0.0003</v>
+        <v>18</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>0.0016</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -2320,13 +2320,13 @@
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H10" s="27" t="n">
-        <v>4373</v>
+        <v>4375</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
@@ -2344,13 +2344,13 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9734</v>
+        <v>9744</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0246</v>
+        <v>0.0257</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
@@ -2358,10 +2358,10 @@
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2741</v>
+        <v>2748</v>
       </c>
       <c r="I11" s="28" t="n">
         <v>7</v>
@@ -2382,13 +2382,13 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7252</v>
+        <v>7340</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>152</v>
+        <v>240</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0214</v>
+        <v>0.0338</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -2396,13 +2396,13 @@
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>832</v>
+        <v>855</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
@@ -2420,13 +2420,13 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6716</v>
+        <v>6730</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0024</v>
+        <v>0.004500000000000001</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
@@ -2434,13 +2434,13 @@
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3114</v>
+        <v>3123</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,13 +2458,13 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6517</v>
+        <v>6539</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0344</v>
+        <v>0.0379</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
@@ -2472,13 +2472,13 @@
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1093</v>
+        <v>1103</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
@@ -2496,13 +2496,13 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4620</v>
+        <v>4613</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>-80</v>
+        <v>-87</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>-0.017</v>
+        <v>-0.0185</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -2510,7 +2510,7 @@
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H15" s="27" t="n">
         <v>815</v>
@@ -2534,13 +2534,13 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4591</v>
+        <v>4599</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-9</v>
+        <v>-1</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.002</v>
+        <v>-0.0002</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -2548,13 +2548,13 @@
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H16" s="27" t="n">
-        <v>1884</v>
+        <v>1890</v>
       </c>
       <c r="I16" s="28" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J16" s="26" t="inlineStr">
         <is>
@@ -2572,13 +2572,13 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2277</v>
+        <v>2276</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>-0.01</v>
+        <v>-0.0104</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
@@ -2586,13 +2586,13 @@
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>2149</v>
+        <v>2151</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -2610,13 +2610,13 @@
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>2220</v>
+        <v>2254</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.0571</v>
+        <v>0.0733</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
@@ -2624,10 +2624,10 @@
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H18" s="27" t="n">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="I18" s="28" t="n">
         <v>2</v>
@@ -2648,13 +2648,13 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1838</v>
+        <v>1841</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0211</v>
+        <v>0.0228</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H19" s="27" t="n">
         <v>176</v>
@@ -2686,13 +2686,13 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1837</v>
+        <v>1838</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0206</v>
+        <v>0.0211</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
@@ -2700,14 +2700,12 @@
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>212</v>
-      </c>
-      <c r="I20" s="28" t="n">
-        <v>0</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="I20" s="28" t="n"/>
       <c r="J20" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2720,17 +2718,17 @@
       </c>
       <c r="B21" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_perth</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1442</v>
+        <v>1463</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-58</v>
-      </c>
-      <c r="E21" s="30" t="n">
-        <v>-0.0387</v>
+        <v>63</v>
+      </c>
+      <c r="E21" s="29" t="n">
+        <v>0.045</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -2738,13 +2736,13 @@
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>1357</v>
+        <v>327</v>
       </c>
       <c r="I21" s="28" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J21" s="26" t="inlineStr">
         <is>
@@ -2758,17 +2756,17 @@
       </c>
       <c r="B22" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>msfitnessaustralia_perth</t>
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1432</v>
+        <v>1439</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>32</v>
-      </c>
-      <c r="E22" s="29" t="n">
-        <v>0.0229</v>
+        <v>-61</v>
+      </c>
+      <c r="E22" s="30" t="n">
+        <v>-0.0407</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
@@ -2776,13 +2774,13 @@
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H22" s="27" t="n">
-        <v>312</v>
+        <v>1357</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J22" s="26" t="inlineStr">
         <is>
@@ -2800,13 +2798,13 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>935</v>
+        <v>947</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.047</v>
+        <v>0.0605</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
@@ -2814,10 +2812,10 @@
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>662</v>
+        <v>676</v>
       </c>
       <c r="I23" s="28" t="n">
         <v>14</v>
@@ -2901,16 +2899,16 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>2220</v>
+        <v>2254</v>
       </c>
       <c r="C2" s="27" t="n">
         <v>2100</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0571</v>
+        <v>0.0733</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
@@ -2918,7 +2916,7 @@
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H2" s="26" t="n">
         <v>17</v>
@@ -2931,16 +2929,16 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>935</v>
+        <v>947</v>
       </c>
       <c r="C3" s="27" t="n">
         <v>893</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.047</v>
+        <v>0.0605</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
@@ -2948,7 +2946,7 @@
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H3" s="26" t="n">
         <v>22</v>
@@ -2957,20 +2955,20 @@
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>icnnewzealand</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6517</v>
+        <v>1463</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>6300</v>
+        <v>1400</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>217</v>
+        <v>63</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0344</v>
+        <v>0.045</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2978,29 +2976,29 @@
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H4" s="26" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" ht="21" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>icnnewzealand</t>
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>57539</v>
+        <v>6539</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>56100</v>
+        <v>6300</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>1439</v>
+        <v>239</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0257</v>
+        <v>0.0379</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
@@ -3008,29 +3006,29 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>anb.australia</t>
+          <t>wnbfaustralia</t>
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>9734</v>
+        <v>7340</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>9500</v>
+        <v>7100</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0246</v>
+        <v>0.0338</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -3038,29 +3036,29 @@
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>1432</v>
+        <v>57884</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>1400</v>
+        <v>56100</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>32</v>
+        <v>1784</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0229</v>
+        <v>0.0318</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
@@ -3068,29 +3066,29 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>wnbfaustralia</t>
+          <t>anb.australia</t>
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>7252</v>
+        <v>9744</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>7100</v>
+        <v>9500</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>152</v>
+        <v>244</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0214</v>
+        <v>0.0257</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -3098,10 +3096,10 @@
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
@@ -3111,16 +3109,16 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>1838</v>
+        <v>1841</v>
       </c>
       <c r="C9" s="27" t="n">
         <v>1800</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0211</v>
+        <v>0.0228</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
@@ -3128,7 +3126,7 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H9" s="26" t="n">
         <v>18</v>
@@ -3137,20 +3135,20 @@
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>icn_nsw</t>
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>1837</v>
+        <v>16135</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>1800</v>
+        <v>15800</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>37</v>
+        <v>335</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0206</v>
+        <v>0.0212</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -3158,29 +3156,29 @@
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>15466</v>
+        <v>1838</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>15200</v>
+        <v>1800</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>266</v>
+        <v>38</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0175</v>
+        <v>0.0211</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
@@ -3188,10 +3186,10 @@
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
@@ -3201,16 +3199,16 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>12893</v>
+        <v>12963</v>
       </c>
       <c r="C12" s="27" t="n">
         <v>12700</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>193</v>
+        <v>263</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0152</v>
+        <v>0.0207</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -3218,7 +3216,7 @@
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H12" s="26" t="n">
         <v>7</v>
@@ -3227,20 +3225,20 @@
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>icn_nsw</t>
+          <t>msfitnessaustralia</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>16036</v>
+        <v>15507</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>15800</v>
+        <v>15200</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>236</v>
+        <v>307</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0149</v>
+        <v>0.0202</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
@@ -3248,10 +3246,10 @@
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
@@ -3261,16 +3259,16 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>18425</v>
+        <v>18529</v>
       </c>
       <c r="C14" s="27" t="n">
         <v>18200</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>225</v>
+        <v>329</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0124</v>
+        <v>0.0181</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
@@ -3278,7 +3276,7 @@
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H14" s="26" t="n">
         <v>2</v>
@@ -3291,16 +3289,16 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>11413</v>
+        <v>11420</v>
       </c>
       <c r="C15" s="27" t="n">
         <v>11300</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.01</v>
+        <v>0.0106</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -3308,7 +3306,7 @@
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H15" s="26" t="n">
         <v>8</v>
@@ -3321,16 +3319,16 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>17835</v>
+        <v>17865</v>
       </c>
       <c r="C16" s="27" t="n">
         <v>17700</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.0076</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -3338,7 +3336,7 @@
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H16" s="26" t="n">
         <v>3</v>
@@ -3351,16 +3349,16 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>6716</v>
+        <v>6730</v>
       </c>
       <c r="C17" s="27" t="n">
         <v>6700</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.0024</v>
+        <v>0.004500000000000001</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
@@ -3368,7 +3366,7 @@
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H17" s="26" t="n">
         <v>12</v>
@@ -3381,16 +3379,16 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>10997</v>
+        <v>11018</v>
       </c>
       <c r="C18" s="27" t="n">
         <v>11000</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>-3</v>
-      </c>
-      <c r="E18" s="30" t="n">
-        <v>-0.0003</v>
+        <v>18</v>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>0.0016</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
@@ -3398,7 +3396,7 @@
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H18" s="26" t="n">
         <v>9</v>
@@ -3411,16 +3409,16 @@
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>4591</v>
+        <v>4599</v>
       </c>
       <c r="C19" s="27" t="n">
         <v>4600</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>-9</v>
+        <v>-1</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>-0.002</v>
+        <v>-0.0002</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
@@ -3428,7 +3426,7 @@
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H19" s="26" t="n">
         <v>15</v>
@@ -3441,16 +3439,16 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>2277</v>
+        <v>2276</v>
       </c>
       <c r="C20" s="27" t="n">
         <v>2300</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>-0.01</v>
+        <v>-0.0104</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
@@ -3458,7 +3456,7 @@
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H20" s="26" t="n">
         <v>16</v>
@@ -3471,16 +3469,16 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>15721</v>
+        <v>15715</v>
       </c>
       <c r="C21" s="27" t="n">
         <v>15900</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-179</v>
+        <v>-185</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.0113</v>
+        <v>-0.0116</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -3488,7 +3486,7 @@
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H21" s="26" t="n">
         <v>5</v>
@@ -3501,16 +3499,16 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>4620</v>
+        <v>4613</v>
       </c>
       <c r="C22" s="27" t="n">
         <v>4700</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-80</v>
+        <v>-87</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.017</v>
+        <v>-0.0185</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
@@ -3518,7 +3516,7 @@
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H22" s="26" t="n">
         <v>14</v>
@@ -3531,16 +3529,16 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>1442</v>
+        <v>1439</v>
       </c>
       <c r="C23" s="27" t="n">
         <v>1500</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-58</v>
+        <v>-61</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>-0.0387</v>
+        <v>-0.0407</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
@@ -3548,10 +3546,10 @@
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H23" s="26" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -3603,14 +3601,14 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>7970</v>
+        <v>8050</v>
       </c>
       <c r="C2" s="28" t="n">
-        <v>168</v>
+        <v>80</v>
       </c>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3621,14 +3619,14 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3335</v>
+        <v>3355</v>
       </c>
       <c r="C3" s="28" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3639,14 +3637,14 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6786</v>
+        <v>6795</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3657,14 +3655,14 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6786</v>
+        <v>6848</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3675,14 +3673,14 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>2970</v>
+        <v>2975</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3693,14 +3691,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3589</v>
+        <v>3596</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3711,14 +3709,14 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4462</v>
+        <v>4468</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3729,14 +3727,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2846</v>
+        <v>2852</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3747,14 +3745,14 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4373</v>
+        <v>4375</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3765,14 +3763,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2741</v>
+        <v>2748</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>7</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3783,14 +3781,14 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>832</v>
+        <v>855</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3801,14 +3799,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3114</v>
+        <v>3123</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3819,14 +3817,14 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1093</v>
+        <v>1103</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3842,7 @@
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3855,14 +3853,14 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>1884</v>
+        <v>1890</v>
       </c>
       <c r="C16" s="28" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3873,14 +3871,14 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>2149</v>
+        <v>2151</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3891,14 +3889,14 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C18" s="28" t="n">
         <v>2</v>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3914,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3927,50 +3925,48 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>212</v>
-      </c>
-      <c r="C20" s="28" t="n">
-        <v>0</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="C20" s="28" t="n"/>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_perth</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>1357</v>
+        <v>327</v>
       </c>
       <c r="C21" s="28" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>msfitnessaustralia_perth</t>
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>312</v>
+        <v>1357</v>
       </c>
       <c r="C22" s="28" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -3981,14 +3977,14 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>662</v>
+        <v>676</v>
       </c>
       <c r="C23" s="28" t="n">
         <v>14</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4033,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4067,7 +4063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D365"/>
+  <dimension ref="A1:D387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11378,6 +11374,446 @@
         </is>
       </c>
     </row>
+    <row r="366" ht="21" customHeight="1">
+      <c r="A366" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B366" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C366" s="27" t="n">
+        <v>9744</v>
+      </c>
+      <c r="D366" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="367" ht="21" customHeight="1">
+      <c r="A367" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B367" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C367" s="27" t="n">
+        <v>2254</v>
+      </c>
+      <c r="D367" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="368" ht="21" customHeight="1">
+      <c r="A368" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B368" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C368" s="27" t="n">
+        <v>1838</v>
+      </c>
+      <c r="D368" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="369" ht="21" customHeight="1">
+      <c r="A369" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B369" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C369" s="27" t="n">
+        <v>1841</v>
+      </c>
+      <c r="D369" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="370" ht="21" customHeight="1">
+      <c r="A370" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B370" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C370" s="27" t="n">
+        <v>4599</v>
+      </c>
+      <c r="D370" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="371" ht="21" customHeight="1">
+      <c r="A371" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B371" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C371" s="27" t="n">
+        <v>16135</v>
+      </c>
+      <c r="D371" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="372" ht="21" customHeight="1">
+      <c r="A372" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B372" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C372" s="27" t="n">
+        <v>1463</v>
+      </c>
+      <c r="D372" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="373" ht="21" customHeight="1">
+      <c r="A373" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B373" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C373" s="27" t="n">
+        <v>6730</v>
+      </c>
+      <c r="D373" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="374" ht="21" customHeight="1">
+      <c r="A374" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B374" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C374" s="27" t="n">
+        <v>2276</v>
+      </c>
+      <c r="D374" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="375" ht="21" customHeight="1">
+      <c r="A375" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B375" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C375" s="27" t="n">
+        <v>12963</v>
+      </c>
+      <c r="D375" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="376" ht="21" customHeight="1">
+      <c r="A376" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B376" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C376" s="27" t="n">
+        <v>11018</v>
+      </c>
+      <c r="D376" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" ht="21" customHeight="1">
+      <c r="A377" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B377" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C377" s="27" t="n">
+        <v>6539</v>
+      </c>
+      <c r="D377" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="378" ht="21" customHeight="1">
+      <c r="A378" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B378" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C378" s="27" t="n">
+        <v>17865</v>
+      </c>
+      <c r="D378" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="379" ht="21" customHeight="1">
+      <c r="A379" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B379" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C379" s="27" t="n">
+        <v>57884</v>
+      </c>
+      <c r="D379" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="380" ht="21" customHeight="1">
+      <c r="A380" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B380" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C380" s="27" t="n">
+        <v>15507</v>
+      </c>
+      <c r="D380" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="381" ht="21" customHeight="1">
+      <c r="A381" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B381" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C381" s="27" t="n">
+        <v>1439</v>
+      </c>
+      <c r="D381" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="382" ht="21" customHeight="1">
+      <c r="A382" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B382" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C382" s="27" t="n">
+        <v>947</v>
+      </c>
+      <c r="D382" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="383" ht="21" customHeight="1">
+      <c r="A383" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B383" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C383" s="27" t="n">
+        <v>15715</v>
+      </c>
+      <c r="D383" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="384" ht="21" customHeight="1">
+      <c r="A384" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B384" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C384" s="27" t="n">
+        <v>18529</v>
+      </c>
+      <c r="D384" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="385" ht="21" customHeight="1">
+      <c r="A385" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B385" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C385" s="27" t="n">
+        <v>11420</v>
+      </c>
+      <c r="D385" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="386" ht="21" customHeight="1">
+      <c r="A386" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B386" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C386" s="27" t="n">
+        <v>7340</v>
+      </c>
+      <c r="D386" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="387" ht="21" customHeight="1">
+      <c r="A387" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B387" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C387" s="27" t="n">
+        <v>4613</v>
+      </c>
+      <c r="D387" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-09-20
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 13 September 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 20 September 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,529</t>
+          <t>18,601</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+1.81%</t>
+          <t>+1.60%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+329 followers • 61 days</t>
+          <t>+293 followers • 33 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>57884</v>
+        <v>58234</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -1272,14 +1272,14 @@
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.0733</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>61d</t>
+          <t>33d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,25 +1295,25 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18529</v>
+        <v>18601</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.0605</v>
+        <v>0.04389999999999999</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>61d</t>
+          <t>33d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,25 +1329,25 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>17865</v>
+        <v>17908</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.045</v>
+        <v>0.0404</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>61d</t>
+          <t>33d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,25 +1363,25 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>16135</v>
+        <v>16217</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>@icnnewzealand</t>
+          <t>@wnbfaustralia</t>
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0379</v>
+        <v>0.0338</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>61d</t>
+          <t>33d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,25 +1397,25 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15715</v>
+        <v>15720</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>@wnbfaustralia</t>
+          <t>@ifbbproleagueoz</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>240</v>
+        <v>1744</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.0338</v>
+        <v>0.0309</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>61d</t>
+          <t>33d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>57884</v>
+        <v>58234</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.0733</v>
+        <v>0.07530000000000001</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,15 +1826,15 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18529</v>
+        <v>18601</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.0605</v>
+        <v>0.04389999999999999</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,15 +1844,15 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17865</v>
+        <v>17908</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.045</v>
+        <v>0.0404</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,15 +1862,15 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16135</v>
+        <v>16217</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>@icnnewzealand</t>
+          <t>@wnbfaustralia</t>
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0379</v>
+        <v>0.0338</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,15 +1880,15 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15715</v>
+        <v>15720</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>@wnbfaustralia</t>
+          <t>@ifbbproleagueoz</t>
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.0338</v>
+        <v>0.0309</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,27 +2002,27 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>57884</v>
+        <v>58234</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>1784</v>
+        <v>1744</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0318</v>
+        <v>0.0309</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H2" s="27" t="n">
-        <v>8050</v>
+        <v>8182</v>
       </c>
       <c r="I2" s="28" t="n">
-        <v>80</v>
+        <v>132</v>
       </c>
       <c r="J2" s="26" t="inlineStr">
         <is>
@@ -2040,27 +2040,27 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18529</v>
+        <v>18601</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>329</v>
+        <v>293</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0181</v>
+        <v>0.016</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3355</v>
+        <v>3378</v>
       </c>
       <c r="I3" s="28" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
@@ -2078,27 +2078,27 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>17865</v>
+        <v>17908</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>165</v>
+        <v>132</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.0074</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6795</v>
+        <v>6839</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2116,27 +2116,27 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>16135</v>
+        <v>16217</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0212</v>
+        <v>0.021</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>6848</v>
+        <v>6907</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
@@ -2154,27 +2154,27 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15715</v>
+        <v>15720</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>-185</v>
+        <v>-158</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>-0.0116</v>
+        <v>-0.01</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>2975</v>
+        <v>2977</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
@@ -2192,24 +2192,24 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15507</v>
+        <v>15534</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>307</v>
+        <v>171</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0202</v>
+        <v>0.0111</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3596</v>
+        <v>3603</v>
       </c>
       <c r="I7" s="28" t="n">
         <v>7</v>
@@ -2230,27 +2230,27 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>12963</v>
+        <v>13019</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>263</v>
+        <v>336</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0207</v>
+        <v>0.0265</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4468</v>
+        <v>4478</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
@@ -2268,27 +2268,27 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11420</v>
+        <v>11437</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>120</v>
+        <v>43</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0106</v>
+        <v>0.0038</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2852</v>
+        <v>2857</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,27 +2306,27 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>11018</v>
+        <v>11088</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0016</v>
+        <v>0.0105</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H10" s="27" t="n">
-        <v>4375</v>
+        <v>4387</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
@@ -2344,27 +2344,27 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9744</v>
+        <v>9759</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>244</v>
+        <v>170</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0257</v>
+        <v>0.0177</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2748</v>
+        <v>2759</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
@@ -2382,27 +2382,27 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7340</v>
+        <v>7433</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E12" s="29" t="n">
         <v>0.0338</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>855</v>
+        <v>897</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
@@ -2420,27 +2420,27 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6730</v>
+        <v>6737</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.004500000000000001</v>
+        <v>0.006</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3123</v>
+        <v>3127</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,27 +2458,27 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6539</v>
+        <v>6560</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>239</v>
+        <v>126</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0379</v>
+        <v>0.0196</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1103</v>
+        <v>1129</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
@@ -2492,31 +2492,31 @@
       </c>
       <c r="B15" s="26" t="inlineStr">
         <is>
-          <t>ynf_australia</t>
+          <t>icn_act</t>
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4613</v>
+        <v>4615</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>-87</v>
-      </c>
-      <c r="E15" s="30" t="n">
-        <v>-0.0185</v>
+        <v>34</v>
+      </c>
+      <c r="E15" s="29" t="n">
+        <v>0.0074</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H15" s="27" t="n">
-        <v>815</v>
+        <v>1899</v>
       </c>
       <c r="I15" s="28" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J15" s="26" t="inlineStr">
         <is>
@@ -2530,31 +2530,31 @@
       </c>
       <c r="B16" s="26" t="inlineStr">
         <is>
-          <t>icn_act</t>
+          <t>ynf_australia</t>
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4599</v>
+        <v>4606</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-1</v>
+        <v>-32</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.0002</v>
+        <v>-0.0069</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H16" s="27" t="n">
-        <v>1890</v>
+        <v>815</v>
       </c>
       <c r="I16" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J16" s="26" t="inlineStr">
         <is>
@@ -2568,31 +2568,31 @@
       </c>
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>icn_tasmania</t>
+          <t>cbrfitexpo</t>
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2276</v>
+        <v>2285</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>-24</v>
-      </c>
-      <c r="E17" s="30" t="n">
-        <v>-0.0104</v>
+        <v>160</v>
+      </c>
+      <c r="E17" s="29" t="n">
+        <v>0.07530000000000001</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>2151</v>
+        <v>338</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -2606,31 +2606,31 @@
       </c>
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>cbrfitexpo</t>
+          <t>icn_tasmania</t>
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>2254</v>
+        <v>2273</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>154</v>
-      </c>
-      <c r="E18" s="29" t="n">
-        <v>0.0733</v>
+        <v>-4</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>-0.0018</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H18" s="27" t="n">
-        <v>337</v>
+        <v>2154</v>
       </c>
       <c r="I18" s="28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J18" s="26" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1841</v>
+        <v>1844</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0228</v>
+        <v>0.0044</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H19" s="27" t="n">
         <v>176</v>
@@ -2686,26 +2686,28 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1838</v>
+        <v>1841</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0211</v>
+        <v>0.006</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>211</v>
-      </c>
-      <c r="I20" s="28" t="n"/>
+        <v>212</v>
+      </c>
+      <c r="I20" s="28" t="n">
+        <v>1</v>
+      </c>
       <c r="J20" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2722,27 +2724,27 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1463</v>
+        <v>1475</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0.045</v>
+        <v>0.04389999999999999</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="I21" s="28" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="J21" s="26" t="inlineStr">
         <is>
@@ -2760,21 +2762,21 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1439</v>
+        <v>1442</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-61</v>
+        <v>-6</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0407</v>
+        <v>-0.004099999999999999</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H22" s="27" t="n">
         <v>1357</v>
@@ -2798,27 +2800,27 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>947</v>
+        <v>952</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.0605</v>
+        <v>0.0404</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>676</v>
+        <v>688</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
@@ -2899,537 +2901,537 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>2254</v>
+        <v>2285</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>2100</v>
+        <v>2125</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0733</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H2" s="26" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_vic</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>947</v>
+        <v>1475</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>893</v>
+        <v>1413</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0605</v>
+        <v>0.04389999999999999</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H3" s="26" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>1463</v>
+        <v>952</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>1400</v>
+        <v>915</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.045</v>
+        <v>0.0404</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H4" s="26" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" ht="21" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>icnnewzealand</t>
+          <t>wnbfaustralia</t>
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6539</v>
+        <v>7433</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>6300</v>
+        <v>7190</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0379</v>
+        <v>0.0338</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>wnbfaustralia</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>7340</v>
+        <v>58234</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>7100</v>
+        <v>56490</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>240</v>
+        <v>1744</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0338</v>
+        <v>0.0309</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>icn_victoria</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>57884</v>
+        <v>13019</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>56100</v>
+        <v>12683</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>1784</v>
+        <v>336</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0318</v>
+        <v>0.0265</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>anb.australia</t>
+          <t>icn_nsw</t>
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>9744</v>
+        <v>16217</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>9500</v>
+        <v>15884</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>244</v>
+        <v>333</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0257</v>
+        <v>0.021</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>icn.indonesia</t>
+          <t>icnnewzealand</t>
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>1841</v>
+        <v>6560</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>1800</v>
+        <v>6434</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>41</v>
+        <v>126</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0228</v>
+        <v>0.0196</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>icn_nsw</t>
+          <t>anb.australia</t>
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>16135</v>
+        <v>9759</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>15800</v>
+        <v>9589</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>335</v>
+        <v>170</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0212</v>
+        <v>0.0177</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>nbaaustralia_official</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>1838</v>
+        <v>18601</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>1800</v>
+        <v>18308</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>38</v>
+        <v>293</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0211</v>
+        <v>0.016</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>icn_victoria</t>
+          <t>msfitnessaustralia</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>12963</v>
+        <v>15534</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>12700</v>
+        <v>15363</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>263</v>
+        <v>171</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0207</v>
+        <v>0.0111</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia</t>
+          <t>icn_wa</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>15507</v>
+        <v>11088</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>15200</v>
+        <v>10973</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>307</v>
+        <v>115</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0202</v>
+        <v>0.0105</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>nbaaustralia_official</t>
+          <t>icnqld</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>18529</v>
+        <v>17908</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>18200</v>
+        <v>17776</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>329</v>
+        <v>132</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0181</v>
+        <v>0.0074</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>pca_australia</t>
+          <t>icn_act</t>
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>11420</v>
+        <v>4615</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>11300</v>
+        <v>4581</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>120</v>
+        <v>34</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0106</v>
+        <v>0.0074</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H15" s="26" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>icnqld</t>
+          <t>icn_sa</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>17865</v>
+        <v>6737</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>17700</v>
+        <v>6697</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>165</v>
+        <v>40</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.006</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H16" s="26" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>icn_sa</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>6730</v>
+        <v>1841</v>
       </c>
       <c r="C17" s="27" t="n">
-        <v>6700</v>
+        <v>1830</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.004500000000000001</v>
+        <v>0.006</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H17" s="26" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>icn_wa</t>
+          <t>icn.indonesia</t>
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>11018</v>
+        <v>1844</v>
       </c>
       <c r="C18" s="27" t="n">
-        <v>11000</v>
+        <v>1836</v>
       </c>
       <c r="D18" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="n">
+        <v>33</v>
+      </c>
+      <c r="H18" s="26" t="n">
         <v>18</v>
-      </c>
-      <c r="E18" s="29" t="n">
-        <v>0.0016</v>
-      </c>
-      <c r="F18" s="26" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="G18" s="26" t="n">
-        <v>61</v>
-      </c>
-      <c r="H18" s="26" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>icn_act</t>
+          <t>pca_australia</t>
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>4599</v>
+        <v>11437</v>
       </c>
       <c r="C19" s="27" t="n">
-        <v>4600</v>
+        <v>11394</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E19" s="30" t="n">
-        <v>-0.0002</v>
+        <v>43</v>
+      </c>
+      <c r="E19" s="29" t="n">
+        <v>0.0038</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
@@ -3439,57 +3441,57 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>2276</v>
+        <v>2273</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>2300</v>
+        <v>2277</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>-24</v>
+        <v>-4</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>-0.0104</v>
+        <v>-0.0018</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H20" s="26" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>nabbaaustralia</t>
+          <t>msfitnessaustralia_perth</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>15715</v>
+        <v>1442</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>15900</v>
+        <v>1448</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-185</v>
+        <v>-6</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.0116</v>
+        <v>-0.004099999999999999</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H21" s="26" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
@@ -3499,57 +3501,57 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>4613</v>
+        <v>4606</v>
       </c>
       <c r="C22" s="27" t="n">
-        <v>4700</v>
+        <v>4638</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-87</v>
+        <v>-32</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0185</v>
+        <v>-0.0069</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H22" s="26" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" ht="21" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_perth</t>
+          <t>nabbaaustralia</t>
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>1439</v>
+        <v>15720</v>
       </c>
       <c r="C23" s="27" t="n">
-        <v>1500</v>
+        <v>15878</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-61</v>
+        <v>-158</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>-0.0407</v>
+        <v>-0.01</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H23" s="26" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3601,14 +3603,14 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>8050</v>
+        <v>8182</v>
       </c>
       <c r="C2" s="28" t="n">
-        <v>80</v>
+        <v>132</v>
       </c>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3619,14 +3621,14 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3355</v>
+        <v>3378</v>
       </c>
       <c r="C3" s="28" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3637,14 +3639,14 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6795</v>
+        <v>6839</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3655,14 +3657,14 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6848</v>
+        <v>6907</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3673,14 +3675,14 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>2975</v>
+        <v>2977</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3691,14 +3693,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3596</v>
+        <v>3603</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>7</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3709,14 +3711,14 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4468</v>
+        <v>4478</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3727,14 +3729,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2852</v>
+        <v>2857</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3745,14 +3747,14 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4375</v>
+        <v>4387</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3763,14 +3765,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2748</v>
+        <v>2759</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3781,14 +3783,14 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>855</v>
+        <v>897</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3799,14 +3801,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3123</v>
+        <v>3127</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3817,86 +3819,86 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1103</v>
+        <v>1129</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>ynf_australia</t>
+          <t>icn_act</t>
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>815</v>
+        <v>1899</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>icn_act</t>
+          <t>ynf_australia</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>1890</v>
+        <v>815</v>
       </c>
       <c r="C16" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>icn_tasmania</t>
+          <t>cbrfitexpo</t>
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>2151</v>
+        <v>338</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>cbrfitexpo</t>
+          <t>icn_tasmania</t>
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>337</v>
+        <v>2154</v>
       </c>
       <c r="C18" s="28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3914,7 +3916,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3925,12 +3927,14 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>211</v>
-      </c>
-      <c r="C20" s="28" t="n"/>
+        <v>212</v>
+      </c>
+      <c r="C20" s="28" t="n">
+        <v>1</v>
+      </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3941,14 +3945,14 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="C21" s="28" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3970,7 @@
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3977,14 +3981,14 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>676</v>
+        <v>688</v>
       </c>
       <c r="C23" s="28" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4037,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4063,7 +4067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D387"/>
+  <dimension ref="A1:D409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11814,6 +11818,446 @@
         </is>
       </c>
     </row>
+    <row r="388" ht="21" customHeight="1">
+      <c r="A388" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B388" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C388" s="27" t="n">
+        <v>9759</v>
+      </c>
+      <c r="D388" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="389" ht="21" customHeight="1">
+      <c r="A389" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B389" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C389" s="27" t="n">
+        <v>2285</v>
+      </c>
+      <c r="D389" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="390" ht="21" customHeight="1">
+      <c r="A390" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B390" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C390" s="27" t="n">
+        <v>1841</v>
+      </c>
+      <c r="D390" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="391" ht="21" customHeight="1">
+      <c r="A391" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B391" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C391" s="27" t="n">
+        <v>1844</v>
+      </c>
+      <c r="D391" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" ht="21" customHeight="1">
+      <c r="A392" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B392" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C392" s="27" t="n">
+        <v>4615</v>
+      </c>
+      <c r="D392" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="393" ht="21" customHeight="1">
+      <c r="A393" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B393" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C393" s="27" t="n">
+        <v>16217</v>
+      </c>
+      <c r="D393" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="394" ht="21" customHeight="1">
+      <c r="A394" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B394" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C394" s="27" t="n">
+        <v>1475</v>
+      </c>
+      <c r="D394" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="395" ht="21" customHeight="1">
+      <c r="A395" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B395" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C395" s="27" t="n">
+        <v>6737</v>
+      </c>
+      <c r="D395" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="396" ht="21" customHeight="1">
+      <c r="A396" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B396" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C396" s="27" t="n">
+        <v>2273</v>
+      </c>
+      <c r="D396" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="397" ht="21" customHeight="1">
+      <c r="A397" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B397" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C397" s="27" t="n">
+        <v>13019</v>
+      </c>
+      <c r="D397" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="398" ht="21" customHeight="1">
+      <c r="A398" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B398" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C398" s="27" t="n">
+        <v>11088</v>
+      </c>
+      <c r="D398" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="399" ht="21" customHeight="1">
+      <c r="A399" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B399" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C399" s="27" t="n">
+        <v>6560</v>
+      </c>
+      <c r="D399" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="400" ht="21" customHeight="1">
+      <c r="A400" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B400" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C400" s="27" t="n">
+        <v>17908</v>
+      </c>
+      <c r="D400" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="401" ht="21" customHeight="1">
+      <c r="A401" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B401" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C401" s="27" t="n">
+        <v>58234</v>
+      </c>
+      <c r="D401" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="402" ht="21" customHeight="1">
+      <c r="A402" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B402" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C402" s="27" t="n">
+        <v>15534</v>
+      </c>
+      <c r="D402" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="403" ht="21" customHeight="1">
+      <c r="A403" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B403" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C403" s="27" t="n">
+        <v>1442</v>
+      </c>
+      <c r="D403" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="404" ht="21" customHeight="1">
+      <c r="A404" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B404" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C404" s="27" t="n">
+        <v>952</v>
+      </c>
+      <c r="D404" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="405" ht="21" customHeight="1">
+      <c r="A405" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B405" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C405" s="27" t="n">
+        <v>15720</v>
+      </c>
+      <c r="D405" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="406" ht="21" customHeight="1">
+      <c r="A406" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B406" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C406" s="27" t="n">
+        <v>18601</v>
+      </c>
+      <c r="D406" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="407" ht="21" customHeight="1">
+      <c r="A407" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B407" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C407" s="27" t="n">
+        <v>11437</v>
+      </c>
+      <c r="D407" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="408" ht="21" customHeight="1">
+      <c r="A408" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B408" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C408" s="27" t="n">
+        <v>7433</v>
+      </c>
+      <c r="D408" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="409" ht="21" customHeight="1">
+      <c r="A409" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B409" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C409" s="27" t="n">
+        <v>4606</v>
+      </c>
+      <c r="D409" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-09-28
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 20 September 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 28 September 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,601</t>
+          <t>18,659</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+1.60%</t>
+          <t>+1.85%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+293 followers • 33 days</t>
+          <t>+339 followers • 36 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>58234</v>
+        <v>58252</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -1272,14 +1272,14 @@
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.06860000000000001</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>33d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,25 +1295,25 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18601</v>
+        <v>18659</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0435</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>33d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,25 +1329,25 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>17908</v>
+        <v>17940</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.0404</v>
+        <v>0.0425</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>33d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>16217</v>
+        <v>16233</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
@@ -1374,14 +1374,14 @@
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>243</v>
+        <v>264</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0338</v>
+        <v>0.0366</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>33d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15720</v>
+        <v>15714</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
@@ -1408,14 +1408,14 @@
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>1744</v>
+        <v>1749</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.0309</v>
+        <v>0.031</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>33d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>58234</v>
+        <v>58252</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.06860000000000001</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,15 +1826,15 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18601</v>
+        <v>18659</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0435</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,15 +1844,15 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17908</v>
+        <v>17940</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.0404</v>
+        <v>0.0425</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16217</v>
+        <v>16233</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0338</v>
+        <v>0.0366</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,7 +1880,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15720</v>
+        <v>15714</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.0309</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,27 +2002,27 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>58234</v>
+        <v>58252</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>1744</v>
+        <v>1749</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0309</v>
+        <v>0.031</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H2" s="27" t="n">
-        <v>8182</v>
+        <v>8186</v>
       </c>
       <c r="I2" s="28" t="n">
-        <v>132</v>
+        <v>4</v>
       </c>
       <c r="J2" s="26" t="inlineStr">
         <is>
@@ -2040,27 +2040,27 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18601</v>
+        <v>18659</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>293</v>
+        <v>339</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.016</v>
+        <v>0.0185</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3378</v>
+        <v>3398</v>
       </c>
       <c r="I3" s="28" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
@@ -2078,27 +2078,27 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>17908</v>
+        <v>17940</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0074</v>
+        <v>0.0086</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6839</v>
+        <v>6854</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2116,27 +2116,27 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>16217</v>
+        <v>16233</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>333</v>
+        <v>290</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.021</v>
+        <v>0.0182</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>6907</v>
+        <v>6928</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
@@ -2154,27 +2154,27 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15720</v>
+        <v>15714</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>-158</v>
+        <v>-122</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>-0.01</v>
+        <v>-0.0077</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>2977</v>
+        <v>2981</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
@@ -2192,27 +2192,27 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15534</v>
+        <v>15551</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0111</v>
+        <v>0.0104</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3603</v>
+        <v>3611</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J7" s="26" t="inlineStr">
         <is>
@@ -2230,24 +2230,24 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>13019</v>
+        <v>13105</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>336</v>
+        <v>382</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0265</v>
+        <v>0.03</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4478</v>
+        <v>4488</v>
       </c>
       <c r="I8" s="28" t="n">
         <v>10</v>
@@ -2268,27 +2268,27 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11437</v>
+        <v>11451</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0038</v>
+        <v>0.0042</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2857</v>
+        <v>2866</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,27 +2306,27 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>11088</v>
+        <v>11133</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0105</v>
+        <v>0.0146</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H10" s="27" t="n">
-        <v>4387</v>
+        <v>4418</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
@@ -2344,27 +2344,27 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9759</v>
+        <v>9779</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>170</v>
+        <v>199</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0177</v>
+        <v>0.0208</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2759</v>
+        <v>2769</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
@@ -2382,27 +2382,27 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7433</v>
+        <v>7468</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>243</v>
+        <v>264</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0338</v>
+        <v>0.0366</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>897</v>
+        <v>916</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
@@ -2420,27 +2420,27 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6737</v>
+        <v>6755</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.006</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3127</v>
+        <v>3130</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,27 +2458,27 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6560</v>
+        <v>6602</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0196</v>
+        <v>0.0165</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1129</v>
+        <v>1140</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
@@ -2496,27 +2496,27 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4615</v>
+        <v>4675</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0074</v>
+        <v>0.0201</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H15" s="27" t="n">
-        <v>1899</v>
+        <v>1923</v>
       </c>
       <c r="I15" s="28" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="J15" s="26" t="inlineStr">
         <is>
@@ -2534,21 +2534,21 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4606</v>
+        <v>4597</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-32</v>
+        <v>-38</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.0069</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H16" s="27" t="n">
         <v>815</v>
@@ -2572,27 +2572,27 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2285</v>
+        <v>2306</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.06860000000000001</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -2610,7 +2610,7 @@
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>2273</v>
+        <v>2274</v>
       </c>
       <c r="D18" s="28" t="n">
         <v>-4</v>
@@ -2620,17 +2620,17 @@
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H18" s="27" t="n">
-        <v>2154</v>
+        <v>2155</v>
       </c>
       <c r="I18" s="28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J18" s="26" t="inlineStr">
         <is>
@@ -2644,32 +2644,30 @@
       </c>
       <c r="B19" s="26" t="inlineStr">
         <is>
-          <t>icn.indonesia</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1844</v>
+        <v>1847</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0044</v>
+        <v>0.0076</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H19" s="27" t="n">
-        <v>176</v>
-      </c>
-      <c r="I19" s="28" t="n">
-        <v>0</v>
-      </c>
+        <v>208</v>
+      </c>
+      <c r="I19" s="28" t="n"/>
       <c r="J19" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2682,31 +2680,31 @@
       </c>
       <c r="B20" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>icn.indonesia</t>
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1841</v>
+        <v>1844</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.006</v>
+        <v>0.0027</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>212</v>
+        <v>176</v>
       </c>
       <c r="I20" s="28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="26" t="inlineStr">
         <is>
@@ -2724,27 +2722,27 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1475</v>
+        <v>1473</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0425</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="I21" s="28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J21" s="26" t="inlineStr">
         <is>
@@ -2762,21 +2760,21 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1442</v>
+        <v>1444</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.004099999999999999</v>
+        <v>-0.0014</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H22" s="27" t="n">
         <v>1357</v>
@@ -2800,27 +2798,27 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>952</v>
+        <v>960</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.0404</v>
+        <v>0.0435</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>688</v>
+        <v>704</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
@@ -2901,24 +2899,24 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>2285</v>
+        <v>2306</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>2125</v>
+        <v>2158</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.06860000000000001</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H2" s="26" t="n">
         <v>16</v>
@@ -2927,61 +2925,61 @@
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>1475</v>
+        <v>960</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>1413</v>
+        <v>920</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0435</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H3" s="26" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_vic</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>952</v>
+        <v>1473</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>915</v>
+        <v>1413</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0404</v>
+        <v>0.0425</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H4" s="26" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" ht="21" customHeight="1">
@@ -2991,24 +2989,24 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>7433</v>
+        <v>7468</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>7190</v>
+        <v>7204</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>243</v>
+        <v>264</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0338</v>
+        <v>0.0366</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>11</v>
@@ -3021,24 +3019,24 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>58234</v>
+        <v>58252</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>56490</v>
+        <v>56503</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>1744</v>
+        <v>1749</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0309</v>
+        <v>0.031</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H6" s="26" t="n">
         <v>1</v>
@@ -3051,24 +3049,24 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>13019</v>
+        <v>13105</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>12683</v>
+        <v>12723</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>336</v>
+        <v>382</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0265</v>
+        <v>0.03</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H7" s="26" t="n">
         <v>7</v>
@@ -3077,151 +3075,151 @@
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>icn_nsw</t>
+          <t>anb.australia</t>
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>16217</v>
+        <v>9779</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>15884</v>
+        <v>9580</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>333</v>
+        <v>199</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.021</v>
+        <v>0.0208</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>icnnewzealand</t>
+          <t>icn_act</t>
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>6560</v>
+        <v>4675</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>6434</v>
+        <v>4583</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>126</v>
+        <v>92</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0196</v>
+        <v>0.0201</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>anb.australia</t>
+          <t>nbaaustralia_official</t>
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>9759</v>
+        <v>18659</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>9589</v>
+        <v>18320</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>170</v>
+        <v>339</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0177</v>
+        <v>0.0185</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>nbaaustralia_official</t>
+          <t>icn_nsw</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>18601</v>
+        <v>16233</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>18308</v>
+        <v>15943</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.016</v>
+        <v>0.0182</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia</t>
+          <t>icnnewzealand</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>15534</v>
+        <v>6602</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>15363</v>
+        <v>6495</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>171</v>
+        <v>107</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0111</v>
+        <v>0.0165</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
@@ -3231,24 +3229,24 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>11088</v>
+        <v>11133</v>
       </c>
       <c r="C13" s="27" t="n">
         <v>10973</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0105</v>
+        <v>0.0146</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H13" s="26" t="n">
         <v>9</v>
@@ -3257,91 +3255,91 @@
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>icnqld</t>
+          <t>msfitnessaustralia</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>17908</v>
+        <v>15551</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>17776</v>
+        <v>15391</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0074</v>
+        <v>0.0104</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>icn_act</t>
+          <t>icn_sa</t>
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>4615</v>
+        <v>6755</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4581</v>
+        <v>6697</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0074</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H15" s="26" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>icn_sa</t>
+          <t>icnqld</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>6737</v>
+        <v>17940</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>6697</v>
+        <v>17787</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>40</v>
+        <v>153</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.006</v>
+        <v>0.0086</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H16" s="26" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
@@ -3351,207 +3349,207 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>1841</v>
+        <v>1847</v>
       </c>
       <c r="C17" s="27" t="n">
-        <v>1830</v>
+        <v>1833</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.006</v>
+        <v>0.0076</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H17" s="26" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>icn.indonesia</t>
+          <t>pca_australia</t>
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>1844</v>
+        <v>11451</v>
       </c>
       <c r="C18" s="27" t="n">
-        <v>1836</v>
+        <v>11403</v>
       </c>
       <c r="D18" s="28" t="n">
+        <v>48</v>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="n">
+        <v>36</v>
+      </c>
+      <c r="H18" s="26" t="n">
         <v>8</v>
-      </c>
-      <c r="E18" s="29" t="n">
-        <v>0.0044</v>
-      </c>
-      <c r="F18" s="26" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="G18" s="26" t="n">
-        <v>33</v>
-      </c>
-      <c r="H18" s="26" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>pca_australia</t>
+          <t>icn.indonesia</t>
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>11437</v>
+        <v>1844</v>
       </c>
       <c r="C19" s="27" t="n">
-        <v>11394</v>
+        <v>1839</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0038</v>
+        <v>0.0027</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>icn_tasmania</t>
+          <t>msfitnessaustralia_perth</t>
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>2273</v>
+        <v>1444</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>2277</v>
+        <v>1446</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>-0.0018</v>
+        <v>-0.0014</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H20" s="26" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_perth</t>
+          <t>icn_tasmania</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>1442</v>
+        <v>2274</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1448</v>
+        <v>2278</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.004099999999999999</v>
+        <v>-0.0018</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H21" s="26" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>ynf_australia</t>
+          <t>nabbaaustralia</t>
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>4606</v>
+        <v>15714</v>
       </c>
       <c r="C22" s="27" t="n">
-        <v>4638</v>
+        <v>15836</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-32</v>
+        <v>-122</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0069</v>
+        <v>-0.0077</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H22" s="26" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" ht="21" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>nabbaaustralia</t>
+          <t>ynf_australia</t>
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>15720</v>
+        <v>4597</v>
       </c>
       <c r="C23" s="27" t="n">
-        <v>15878</v>
+        <v>4635</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-158</v>
+        <v>-38</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>-0.01</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H23" s="26" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3603,14 +3601,14 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>8182</v>
+        <v>8186</v>
       </c>
       <c r="C2" s="28" t="n">
-        <v>132</v>
+        <v>4</v>
       </c>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3621,14 +3619,14 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3378</v>
+        <v>3398</v>
       </c>
       <c r="C3" s="28" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3639,14 +3637,14 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6839</v>
+        <v>6854</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3657,14 +3655,14 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6907</v>
+        <v>6928</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3675,14 +3673,14 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>2977</v>
+        <v>2981</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3693,14 +3691,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3603</v>
+        <v>3611</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3711,14 +3709,14 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4478</v>
+        <v>4488</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>10</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3729,14 +3727,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2857</v>
+        <v>2866</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3747,14 +3745,14 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4387</v>
+        <v>4418</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3765,14 +3763,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2759</v>
+        <v>2769</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3783,14 +3781,14 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>897</v>
+        <v>916</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3801,14 +3799,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3127</v>
+        <v>3130</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3819,14 +3817,14 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1129</v>
+        <v>1140</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3837,14 +3835,14 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>1899</v>
+        <v>1923</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3860,7 @@
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3873,14 +3871,14 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3891,50 +3889,48 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>2154</v>
+        <v>2155</v>
       </c>
       <c r="C18" s="28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>icn.indonesia</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>176</v>
-      </c>
-      <c r="C19" s="28" t="n">
-        <v>0</v>
-      </c>
+        <v>208</v>
+      </c>
+      <c r="C19" s="28" t="n"/>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>icn.indonesia</t>
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>212</v>
+        <v>176</v>
       </c>
       <c r="C20" s="28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3945,14 +3941,14 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C21" s="28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3970,7 +3966,7 @@
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3981,14 +3977,14 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>688</v>
+        <v>704</v>
       </c>
       <c r="C23" s="28" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4033,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4067,7 +4063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D409"/>
+  <dimension ref="A1:D431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12258,6 +12254,446 @@
         </is>
       </c>
     </row>
+    <row r="410" ht="21" customHeight="1">
+      <c r="A410" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B410" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C410" s="27" t="n">
+        <v>9779</v>
+      </c>
+      <c r="D410" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="411" ht="21" customHeight="1">
+      <c r="A411" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B411" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C411" s="27" t="n">
+        <v>2306</v>
+      </c>
+      <c r="D411" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="412" ht="21" customHeight="1">
+      <c r="A412" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B412" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C412" s="27" t="n">
+        <v>1847</v>
+      </c>
+      <c r="D412" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="413" ht="21" customHeight="1">
+      <c r="A413" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B413" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C413" s="27" t="n">
+        <v>1844</v>
+      </c>
+      <c r="D413" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="414" ht="21" customHeight="1">
+      <c r="A414" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B414" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C414" s="27" t="n">
+        <v>4675</v>
+      </c>
+      <c r="D414" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="415" ht="21" customHeight="1">
+      <c r="A415" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B415" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C415" s="27" t="n">
+        <v>16233</v>
+      </c>
+      <c r="D415" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="416" ht="21" customHeight="1">
+      <c r="A416" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B416" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C416" s="27" t="n">
+        <v>1473</v>
+      </c>
+      <c r="D416" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="417" ht="21" customHeight="1">
+      <c r="A417" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B417" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C417" s="27" t="n">
+        <v>6755</v>
+      </c>
+      <c r="D417" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="418" ht="21" customHeight="1">
+      <c r="A418" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B418" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C418" s="27" t="n">
+        <v>2274</v>
+      </c>
+      <c r="D418" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="419" ht="21" customHeight="1">
+      <c r="A419" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B419" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C419" s="27" t="n">
+        <v>13105</v>
+      </c>
+      <c r="D419" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="420" ht="21" customHeight="1">
+      <c r="A420" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B420" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C420" s="27" t="n">
+        <v>11133</v>
+      </c>
+      <c r="D420" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="421" ht="21" customHeight="1">
+      <c r="A421" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B421" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C421" s="27" t="n">
+        <v>6602</v>
+      </c>
+      <c r="D421" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="422" ht="21" customHeight="1">
+      <c r="A422" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B422" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C422" s="27" t="n">
+        <v>17940</v>
+      </c>
+      <c r="D422" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="423" ht="21" customHeight="1">
+      <c r="A423" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B423" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C423" s="27" t="n">
+        <v>58252</v>
+      </c>
+      <c r="D423" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="424" ht="21" customHeight="1">
+      <c r="A424" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B424" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C424" s="27" t="n">
+        <v>15551</v>
+      </c>
+      <c r="D424" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="425" ht="21" customHeight="1">
+      <c r="A425" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B425" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C425" s="27" t="n">
+        <v>1444</v>
+      </c>
+      <c r="D425" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="426" ht="21" customHeight="1">
+      <c r="A426" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B426" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C426" s="27" t="n">
+        <v>960</v>
+      </c>
+      <c r="D426" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="427" ht="21" customHeight="1">
+      <c r="A427" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B427" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C427" s="27" t="n">
+        <v>15714</v>
+      </c>
+      <c r="D427" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="428" ht="21" customHeight="1">
+      <c r="A428" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B428" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C428" s="27" t="n">
+        <v>18659</v>
+      </c>
+      <c r="D428" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="429" ht="21" customHeight="1">
+      <c r="A429" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B429" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C429" s="27" t="n">
+        <v>11451</v>
+      </c>
+      <c r="D429" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="430" ht="21" customHeight="1">
+      <c r="A430" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B430" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C430" s="27" t="n">
+        <v>7468</v>
+      </c>
+      <c r="D430" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="431" ht="21" customHeight="1">
+      <c r="A431" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B431" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C431" s="27" t="n">
+        <v>4597</v>
+      </c>
+      <c r="D431" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-10-05
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 28 September 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 05 October 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,659</t>
+          <t>18,678</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+339 followers • 36 days</t>
+          <t>+339 followers • 35 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>58252</v>
+        <v>58237</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -1272,14 +1272,14 @@
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>148</v>
+        <v>272</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.06860000000000001</v>
+        <v>0.1252</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,25 +1295,25 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18659</v>
+        <v>18678</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.0435</v>
+        <v>0.0488</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,25 +1329,25 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>17940</v>
+        <v>18029</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.0425</v>
+        <v>0.0464</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>16233</v>
+        <v>16311</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
@@ -1374,14 +1374,14 @@
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>264</v>
+        <v>287</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0366</v>
+        <v>0.0398</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,25 +1397,25 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15714</v>
+        <v>15807</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>@ifbbproleagueoz</t>
+          <t>@icn_victoria</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>1749</v>
+        <v>394</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.031</v>
+        <v>0.0308</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>58252</v>
+        <v>58237</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.06860000000000001</v>
+        <v>0.1252</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,15 +1826,15 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18659</v>
+        <v>18678</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.0435</v>
+        <v>0.0488</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,15 +1844,15 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17940</v>
+        <v>18029</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.0425</v>
+        <v>0.0464</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16233</v>
+        <v>16311</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0366</v>
+        <v>0.0398</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,15 +1880,15 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15714</v>
+        <v>15807</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>@ifbbproleagueoz</t>
+          <t>@icn_victoria</t>
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.031</v>
+        <v>0.0308</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,27 +2002,27 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>58252</v>
+        <v>58237</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>1749</v>
+        <v>1399</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.031</v>
+        <v>0.0246</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H2" s="27" t="n">
         <v>8186</v>
       </c>
       <c r="I2" s="28" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J2" s="26" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18659</v>
+        <v>18678</v>
       </c>
       <c r="D3" s="28" t="n">
         <v>339</v>
@@ -2050,17 +2050,17 @@
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3398</v>
+        <v>3409</v>
       </c>
       <c r="I3" s="28" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
@@ -2078,27 +2078,27 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>17940</v>
+        <v>18029</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>153</v>
+        <v>236</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0086</v>
+        <v>0.0133</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6854</v>
+        <v>6895</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2116,27 +2116,27 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>16233</v>
+        <v>16311</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0182</v>
+        <v>0.0184</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>6928</v>
+        <v>7004</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
@@ -2154,27 +2154,27 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15714</v>
+        <v>15807</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>-122</v>
-      </c>
-      <c r="E6" s="30" t="n">
-        <v>-0.0077</v>
+        <v>14</v>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>0.0009</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>2981</v>
+        <v>3024</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
@@ -2192,27 +2192,27 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15551</v>
+        <v>15588</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0104</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3611</v>
+        <v>3625</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="J7" s="26" t="inlineStr">
         <is>
@@ -2230,27 +2230,27 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>13105</v>
+        <v>13195</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.03</v>
+        <v>0.0308</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4488</v>
+        <v>4491</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
@@ -2268,27 +2268,27 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11451</v>
+        <v>11495</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0042</v>
+        <v>0.0074</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2866</v>
+        <v>2892</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,27 +2306,27 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>11133</v>
+        <v>11176</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>160</v>
+        <v>198</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0146</v>
+        <v>0.018</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="H10" s="27" t="n">
+        <v>4454</v>
+      </c>
+      <c r="I10" s="28" t="n">
         <v>36</v>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>4418</v>
-      </c>
-      <c r="I10" s="28" t="n">
-        <v>31</v>
       </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
@@ -2344,27 +2344,27 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9779</v>
+        <v>9832</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>199</v>
+        <v>115</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0208</v>
+        <v>0.0118</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2769</v>
+        <v>2792</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
@@ -2382,27 +2382,27 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7468</v>
+        <v>7498</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>264</v>
+        <v>287</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0366</v>
+        <v>0.0398</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>916</v>
+        <v>922</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
@@ -2420,27 +2420,27 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6755</v>
+        <v>6876</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>58</v>
+        <v>167</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0249</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3130</v>
+        <v>3231</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>3</v>
+        <v>101</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6602</v>
+        <v>6605</v>
       </c>
       <c r="D14" s="28" t="n">
         <v>107</v>
@@ -2468,17 +2468,17 @@
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1140</v>
+        <v>1168</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
@@ -2496,27 +2496,27 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4675</v>
+        <v>4690</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0201</v>
+        <v>0.0222</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H15" s="27" t="n">
-        <v>1923</v>
+        <v>1950</v>
       </c>
       <c r="I15" s="28" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J15" s="26" t="inlineStr">
         <is>
@@ -2534,28 +2534,26 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4597</v>
+        <v>4590</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-38</v>
+        <v>-39</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H16" s="27" t="n">
-        <v>815</v>
-      </c>
-      <c r="I16" s="28" t="n">
-        <v>0</v>
-      </c>
+        <v>814</v>
+      </c>
+      <c r="I16" s="28" t="n"/>
       <c r="J16" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2572,27 +2570,27 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2306</v>
+        <v>2445</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>148</v>
+        <v>272</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.06860000000000001</v>
+        <v>0.1252</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>346</v>
+        <v>363</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -2610,28 +2608,26 @@
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>2274</v>
+        <v>2270</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>-0.0018</v>
+        <v>-0.0026</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H18" s="27" t="n">
-        <v>2155</v>
-      </c>
-      <c r="I18" s="28" t="n">
-        <v>1</v>
-      </c>
+        <v>2125</v>
+      </c>
+      <c r="I18" s="28" t="n"/>
       <c r="J18" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2648,26 +2644,28 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1847</v>
+        <v>1850</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0076</v>
+        <v>0.0115</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H19" s="27" t="n">
         <v>208</v>
       </c>
-      <c r="I19" s="28" t="n"/>
+      <c r="I19" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="J19" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2684,21 +2682,21 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1844</v>
+        <v>1845</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0027</v>
+        <v>0.0011</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H20" s="27" t="n">
         <v>176</v>
@@ -2722,27 +2720,27 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1473</v>
+        <v>1483</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0.0425</v>
+        <v>0.0488</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="I21" s="28" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J21" s="26" t="inlineStr">
         <is>
@@ -2760,21 +2758,21 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1444</v>
+        <v>1443</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0014</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H22" s="27" t="n">
         <v>1357</v>
@@ -2798,27 +2796,27 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>960</v>
+        <v>970</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.0435</v>
+        <v>0.0464</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>704</v>
+        <v>727</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
@@ -2899,24 +2897,24 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>2306</v>
+        <v>2445</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>2158</v>
+        <v>2173</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>148</v>
+        <v>272</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.06860000000000001</v>
+        <v>0.1252</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H2" s="26" t="n">
         <v>16</v>
@@ -2925,61 +2923,61 @@
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_vic</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>960</v>
+        <v>1483</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>920</v>
+        <v>1414</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0435</v>
+        <v>0.0488</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H3" s="26" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>1473</v>
+        <v>970</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>1413</v>
+        <v>927</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0425</v>
+        <v>0.0464</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H4" s="26" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" ht="21" customHeight="1">
@@ -2989,24 +2987,24 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>7468</v>
+        <v>7498</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>7204</v>
+        <v>7211</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>264</v>
+        <v>287</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0366</v>
+        <v>0.0398</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>11</v>
@@ -3015,91 +3013,91 @@
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>icn_victoria</t>
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>58252</v>
+        <v>13195</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>56503</v>
+        <v>12801</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>1749</v>
+        <v>394</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.031</v>
+        <v>0.0308</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>icn_victoria</t>
+          <t>icn_sa</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>13105</v>
+        <v>6876</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>12723</v>
+        <v>6709</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>382</v>
+        <v>167</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.03</v>
+        <v>0.0249</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>anb.australia</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>9779</v>
+        <v>58237</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>9580</v>
+        <v>56838</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>199</v>
+        <v>1399</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0208</v>
+        <v>0.0246</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
@@ -3109,24 +3107,24 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>4675</v>
+        <v>4690</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>4583</v>
+        <v>4588</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0201</v>
+        <v>0.0222</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H9" s="26" t="n">
         <v>14</v>
@@ -3139,10 +3137,10 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>18659</v>
+        <v>18678</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>18320</v>
+        <v>18339</v>
       </c>
       <c r="D10" s="28" t="n">
         <v>339</v>
@@ -3152,11 +3150,11 @@
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H10" s="26" t="n">
         <v>2</v>
@@ -3169,24 +3167,24 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>16233</v>
+        <v>16311</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>15943</v>
+        <v>16017</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0182</v>
+        <v>0.0184</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H11" s="26" t="n">
         <v>4</v>
@@ -3195,181 +3193,181 @@
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>icnnewzealand</t>
+          <t>icn_wa</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>6602</v>
+        <v>11176</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>6495</v>
+        <v>10978</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>107</v>
+        <v>198</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0165</v>
+        <v>0.018</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>icn_wa</t>
+          <t>icnnewzealand</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>11133</v>
+        <v>6605</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>10973</v>
+        <v>6498</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>160</v>
+        <v>107</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0146</v>
+        <v>0.0165</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia</t>
+          <t>icnqld</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>15551</v>
+        <v>18029</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>15391</v>
+        <v>17793</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>160</v>
+        <v>236</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0104</v>
+        <v>0.0133</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>icn_sa</t>
+          <t>anb.australia</t>
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>6755</v>
+        <v>9832</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>6697</v>
+        <v>9717</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>58</v>
+        <v>115</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0118</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H15" s="26" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>icnqld</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>17940</v>
+        <v>1850</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>17787</v>
+        <v>1829</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>153</v>
+        <v>21</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.0086</v>
+        <v>0.0115</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H16" s="26" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>msfitnessaustralia</t>
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>1847</v>
+        <v>15588</v>
       </c>
       <c r="C17" s="27" t="n">
-        <v>1833</v>
+        <v>15440</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>14</v>
+        <v>148</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.0076</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H17" s="26" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
@@ -3379,24 +3377,24 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>11451</v>
+        <v>11495</v>
       </c>
       <c r="C18" s="27" t="n">
-        <v>11403</v>
+        <v>11410</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.0042</v>
+        <v>0.0074</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H18" s="26" t="n">
         <v>8</v>
@@ -3409,24 +3407,24 @@
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>1844</v>
+        <v>1845</v>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1839</v>
+        <v>1843</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0027</v>
+        <v>0.0011</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H19" s="26" t="n">
         <v>19</v>
@@ -3435,91 +3433,91 @@
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_perth</t>
+          <t>nabbaaustralia</t>
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>1444</v>
+        <v>15807</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1446</v>
+        <v>15793</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>-2</v>
-      </c>
-      <c r="E20" s="30" t="n">
-        <v>-0.0014</v>
+        <v>14</v>
+      </c>
+      <c r="E20" s="29" t="n">
+        <v>0.0009</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H20" s="26" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>icn_tasmania</t>
+          <t>msfitnessaustralia_perth</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>2274</v>
+        <v>1443</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>2278</v>
+        <v>1444</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.0018</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H21" s="26" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>nabbaaustralia</t>
+          <t>icn_tasmania</t>
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>15714</v>
+        <v>2270</v>
       </c>
       <c r="C22" s="27" t="n">
-        <v>15836</v>
+        <v>2276</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-122</v>
+        <v>-6</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0077</v>
+        <v>-0.0026</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H22" s="26" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" ht="21" customHeight="1">
@@ -3529,24 +3527,24 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>4597</v>
+        <v>4590</v>
       </c>
       <c r="C23" s="27" t="n">
-        <v>4635</v>
+        <v>4629</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-38</v>
+        <v>-39</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H23" s="26" t="n">
         <v>15</v>
@@ -3604,11 +3602,11 @@
         <v>8186</v>
       </c>
       <c r="C2" s="28" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3619,14 +3617,14 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3398</v>
+        <v>3409</v>
       </c>
       <c r="C3" s="28" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3637,14 +3635,14 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6854</v>
+        <v>6895</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3655,14 +3653,14 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6928</v>
+        <v>7004</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3673,14 +3671,14 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>2981</v>
+        <v>3024</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3691,14 +3689,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3611</v>
+        <v>3625</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3709,14 +3707,14 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4488</v>
+        <v>4491</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3727,14 +3725,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2866</v>
+        <v>2892</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3745,14 +3743,14 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4418</v>
+        <v>4454</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3763,14 +3761,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2769</v>
+        <v>2792</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3781,14 +3779,14 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>916</v>
+        <v>922</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3799,14 +3797,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3130</v>
+        <v>3231</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>3</v>
+        <v>101</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3817,14 +3815,14 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1140</v>
+        <v>1168</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3835,14 +3833,14 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>1923</v>
+        <v>1950</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3853,14 +3851,12 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>815</v>
-      </c>
-      <c r="C16" s="28" t="n">
-        <v>0</v>
-      </c>
+        <v>814</v>
+      </c>
+      <c r="C16" s="28" t="n"/>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3871,14 +3867,14 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>346</v>
+        <v>363</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3889,14 +3885,12 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>2155</v>
-      </c>
-      <c r="C18" s="28" t="n">
-        <v>1</v>
-      </c>
+        <v>2125</v>
+      </c>
+      <c r="C18" s="28" t="n"/>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3909,10 +3903,12 @@
       <c r="B19" s="27" t="n">
         <v>208</v>
       </c>
-      <c r="C19" s="28" t="n"/>
+      <c r="C19" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3926,7 @@
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3941,14 +3937,14 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="C21" s="28" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3962,7 @@
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -3977,14 +3973,14 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>704</v>
+        <v>727</v>
       </c>
       <c r="C23" s="28" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4029,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4063,7 +4059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D431"/>
+  <dimension ref="A1:D453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12694,6 +12690,446 @@
         </is>
       </c>
     </row>
+    <row r="432" ht="21" customHeight="1">
+      <c r="A432" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B432" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C432" s="27" t="n">
+        <v>9832</v>
+      </c>
+      <c r="D432" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="433" ht="21" customHeight="1">
+      <c r="A433" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B433" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C433" s="27" t="n">
+        <v>2445</v>
+      </c>
+      <c r="D433" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="434" ht="21" customHeight="1">
+      <c r="A434" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B434" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C434" s="27" t="n">
+        <v>1850</v>
+      </c>
+      <c r="D434" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="435" ht="21" customHeight="1">
+      <c r="A435" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B435" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C435" s="27" t="n">
+        <v>1845</v>
+      </c>
+      <c r="D435" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="436" ht="21" customHeight="1">
+      <c r="A436" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B436" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C436" s="27" t="n">
+        <v>4690</v>
+      </c>
+      <c r="D436" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="437" ht="21" customHeight="1">
+      <c r="A437" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B437" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C437" s="27" t="n">
+        <v>16311</v>
+      </c>
+      <c r="D437" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="438" ht="21" customHeight="1">
+      <c r="A438" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B438" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C438" s="27" t="n">
+        <v>1483</v>
+      </c>
+      <c r="D438" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="439" ht="21" customHeight="1">
+      <c r="A439" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B439" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C439" s="27" t="n">
+        <v>6876</v>
+      </c>
+      <c r="D439" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="440" ht="21" customHeight="1">
+      <c r="A440" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B440" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C440" s="27" t="n">
+        <v>2270</v>
+      </c>
+      <c r="D440" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="441" ht="21" customHeight="1">
+      <c r="A441" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B441" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C441" s="27" t="n">
+        <v>13195</v>
+      </c>
+      <c r="D441" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="442" ht="21" customHeight="1">
+      <c r="A442" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B442" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C442" s="27" t="n">
+        <v>11176</v>
+      </c>
+      <c r="D442" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="443" ht="21" customHeight="1">
+      <c r="A443" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B443" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C443" s="27" t="n">
+        <v>6605</v>
+      </c>
+      <c r="D443" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="444" ht="21" customHeight="1">
+      <c r="A444" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B444" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C444" s="27" t="n">
+        <v>18029</v>
+      </c>
+      <c r="D444" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="445" ht="21" customHeight="1">
+      <c r="A445" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B445" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C445" s="27" t="n">
+        <v>58237</v>
+      </c>
+      <c r="D445" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="446" ht="21" customHeight="1">
+      <c r="A446" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B446" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C446" s="27" t="n">
+        <v>15588</v>
+      </c>
+      <c r="D446" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="447" ht="21" customHeight="1">
+      <c r="A447" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B447" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C447" s="27" t="n">
+        <v>1443</v>
+      </c>
+      <c r="D447" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="448" ht="21" customHeight="1">
+      <c r="A448" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B448" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C448" s="27" t="n">
+        <v>970</v>
+      </c>
+      <c r="D448" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="449" ht="21" customHeight="1">
+      <c r="A449" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B449" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C449" s="27" t="n">
+        <v>15807</v>
+      </c>
+      <c r="D449" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="450" ht="21" customHeight="1">
+      <c r="A450" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B450" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C450" s="27" t="n">
+        <v>18678</v>
+      </c>
+      <c r="D450" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="451" ht="21" customHeight="1">
+      <c r="A451" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B451" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C451" s="27" t="n">
+        <v>11495</v>
+      </c>
+      <c r="D451" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="452" ht="21" customHeight="1">
+      <c r="A452" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B452" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C452" s="27" t="n">
+        <v>7498</v>
+      </c>
+      <c r="D452" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="453" ht="21" customHeight="1">
+      <c r="A453" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B453" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C453" s="27" t="n">
+        <v>4590</v>
+      </c>
+      <c r="D453" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-10-12
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 05 October 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 12 October 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,678</t>
+          <t>18,778</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+1.85%</t>
+          <t>+1.92%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+339 followers • 35 days</t>
+          <t>+353 followers • 36 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>58237</v>
+        <v>58222</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -1272,14 +1272,14 @@
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>272</v>
+        <v>430</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.1252</v>
+        <v>0.1937</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,25 +1295,25 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18678</v>
+        <v>18778</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.0488</v>
+        <v>0.0417</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,25 +1329,25 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>18029</v>
+        <v>18063</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.0464</v>
+        <v>0.0384</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>16311</v>
+        <v>16320</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
@@ -1374,14 +1374,14 @@
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>287</v>
+        <v>253</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0398</v>
+        <v>0.0349</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,25 +1397,25 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15807</v>
+        <v>15804</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>@icn_victoria</t>
+          <t>@icn_sa</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>394</v>
+        <v>187</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.0308</v>
+        <v>0.0278</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>36d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>58237</v>
+        <v>58222</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.1252</v>
+        <v>0.1937</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,15 +1826,15 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18678</v>
+        <v>18778</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.0488</v>
+        <v>0.0417</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,15 +1844,15 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>18029</v>
+        <v>18063</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.0464</v>
+        <v>0.0384</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16311</v>
+        <v>16320</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0398</v>
+        <v>0.0349</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,15 +1880,15 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15807</v>
+        <v>15804</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>@icn_victoria</t>
+          <t>@icn_sa</t>
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.0308</v>
+        <v>0.0278</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,21 +2002,21 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>58237</v>
+        <v>58222</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>1399</v>
+        <v>683</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0246</v>
+        <v>0.0119</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H2" s="27" t="n">
         <v>8186</v>
@@ -2040,27 +2040,27 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18678</v>
+        <v>18778</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>339</v>
+        <v>353</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0185</v>
+        <v>0.0192</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3409</v>
+        <v>3440</v>
       </c>
       <c r="I3" s="28" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
@@ -2078,27 +2078,27 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>18029</v>
+        <v>18063</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0133</v>
+        <v>0.0128</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6895</v>
+        <v>6927</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2116,27 +2116,27 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>16311</v>
+        <v>16320</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0184</v>
+        <v>0.0177</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>7004</v>
+        <v>7042</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
@@ -2154,27 +2154,27 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15807</v>
+        <v>15804</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0009</v>
+        <v>0.0053</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>3024</v>
+        <v>3060</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
@@ -2192,27 +2192,27 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15588</v>
+        <v>15579</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>148</v>
+        <v>113</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0073</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3625</v>
+        <v>3652</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="J7" s="26" t="inlineStr">
         <is>
@@ -2230,27 +2230,27 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>13195</v>
+        <v>13226</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>394</v>
+        <v>333</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0308</v>
+        <v>0.0258</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4491</v>
+        <v>4510</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
@@ -2268,27 +2268,27 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11495</v>
+        <v>11519</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0074</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2892</v>
+        <v>2898</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,27 +2306,27 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>11176</v>
+        <v>11184</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H10" s="27" t="n">
-        <v>4454</v>
+        <v>4460</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
@@ -2344,24 +2344,24 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9832</v>
+        <v>9846</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0118</v>
+        <v>0.0115</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2792</v>
+        <v>2815</v>
       </c>
       <c r="I11" s="28" t="n">
         <v>23</v>
@@ -2382,27 +2382,27 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7498</v>
+        <v>7505</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>287</v>
+        <v>253</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0398</v>
+        <v>0.0349</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H12" s="27" t="n">
         <v>922</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
@@ -2420,27 +2420,27 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6876</v>
+        <v>6903</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0249</v>
+        <v>0.0278</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3231</v>
+        <v>3251</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>101</v>
+        <v>20</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,27 +2458,27 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6605</v>
+        <v>6610</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0165</v>
+        <v>0.0143</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1168</v>
+        <v>1173</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
@@ -2496,27 +2496,27 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4690</v>
+        <v>4702</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0222</v>
+        <v>0.0242</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H15" s="27" t="n">
-        <v>1950</v>
+        <v>1955</v>
       </c>
       <c r="I15" s="28" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="J15" s="26" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4590</v>
+        <v>4581</v>
       </c>
       <c r="D16" s="28" t="n">
         <v>-39</v>
@@ -2544,16 +2544,18 @@
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H16" s="27" t="n">
         <v>814</v>
       </c>
-      <c r="I16" s="28" t="n"/>
+      <c r="I16" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="J16" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2570,27 +2572,27 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2445</v>
+        <v>2650</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>272</v>
+        <v>430</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.1252</v>
+        <v>0.1937</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>363</v>
+        <v>396</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -2608,26 +2610,28 @@
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>2270</v>
+        <v>2276</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>-0.0026</v>
+        <v>-0.0004</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H18" s="27" t="n">
-        <v>2125</v>
-      </c>
-      <c r="I18" s="28" t="n"/>
+        <v>2127</v>
+      </c>
+      <c r="I18" s="28" t="n">
+        <v>2</v>
+      </c>
       <c r="J18" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2644,21 +2648,21 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1850</v>
+        <v>1852</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0115</v>
+        <v>0.008199999999999999</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H19" s="27" t="n">
         <v>208</v>
@@ -2682,21 +2686,21 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1845</v>
+        <v>1838</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0011</v>
+        <v>0</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H20" s="27" t="n">
         <v>176</v>
@@ -2720,27 +2724,27 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1483</v>
+        <v>1487</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0.0488</v>
+        <v>0.0384</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="I21" s="28" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J21" s="26" t="inlineStr">
         <is>
@@ -2761,18 +2765,18 @@
         <v>1443</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E22" s="30" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>1</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>0.0007000000000000001</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H22" s="27" t="n">
         <v>1357</v>
@@ -2796,27 +2800,27 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.0464</v>
+        <v>0.0417</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
@@ -2897,24 +2901,24 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>2445</v>
+        <v>2650</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>2173</v>
+        <v>2220</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>272</v>
+        <v>430</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.1252</v>
+        <v>0.1937</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H2" s="26" t="n">
         <v>16</v>
@@ -2923,61 +2927,61 @@
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>1483</v>
+        <v>974</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>1414</v>
+        <v>935</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0488</v>
+        <v>0.0417</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" s="26" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_vic</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>970</v>
+        <v>1487</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>927</v>
+        <v>1432</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0464</v>
+        <v>0.0384</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H4" s="26" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" ht="21" customHeight="1">
@@ -2987,24 +2991,24 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>7498</v>
+        <v>7505</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>7211</v>
+        <v>7252</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>287</v>
+        <v>253</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0398</v>
+        <v>0.0349</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>11</v>
@@ -3013,271 +3017,271 @@
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>icn_victoria</t>
+          <t>icn_sa</t>
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>13195</v>
+        <v>6903</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>12801</v>
+        <v>6716</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>394</v>
+        <v>187</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0308</v>
+        <v>0.0278</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>icn_sa</t>
+          <t>icn_victoria</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>6876</v>
+        <v>13226</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>6709</v>
+        <v>12893</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>167</v>
+        <v>333</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0249</v>
+        <v>0.0258</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>icn_act</t>
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>58237</v>
+        <v>4702</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>56838</v>
+        <v>4591</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>1399</v>
+        <v>111</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0246</v>
+        <v>0.0242</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>icn_act</t>
+          <t>nbaaustralia_official</t>
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>4690</v>
+        <v>18778</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>4588</v>
+        <v>18425</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>102</v>
+        <v>353</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0222</v>
+        <v>0.0192</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>nbaaustralia_official</t>
+          <t>icn_nsw</t>
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>18678</v>
+        <v>16320</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>18339</v>
+        <v>16036</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>339</v>
+        <v>284</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0185</v>
+        <v>0.0177</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>icn_nsw</t>
+          <t>icn_wa</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>16311</v>
+        <v>11184</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>16017</v>
+        <v>10997</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>294</v>
+        <v>187</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0184</v>
+        <v>0.017</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>icn_wa</t>
+          <t>icnnewzealand</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>11176</v>
+        <v>6610</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>10978</v>
+        <v>6517</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>198</v>
+        <v>93</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.018</v>
+        <v>0.0143</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>icnnewzealand</t>
+          <t>icnqld</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>6605</v>
+        <v>18063</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6498</v>
+        <v>17835</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>107</v>
+        <v>228</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0165</v>
+        <v>0.0128</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>icnqld</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>18029</v>
+        <v>58222</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>17793</v>
+        <v>57539</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>236</v>
+        <v>683</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0133</v>
+        <v>0.0119</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
@@ -3287,24 +3291,24 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>9832</v>
+        <v>9846</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>9717</v>
+        <v>9734</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0118</v>
+        <v>0.0115</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H15" s="26" t="n">
         <v>10</v>
@@ -3313,181 +3317,181 @@
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>pca_australia</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>1850</v>
+        <v>11519</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>1829</v>
+        <v>11413</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>21</v>
+        <v>106</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.0115</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H16" s="26" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>15588</v>
+        <v>1852</v>
       </c>
       <c r="C17" s="27" t="n">
-        <v>15440</v>
+        <v>1837</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>148</v>
+        <v>15</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.008199999999999999</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H17" s="26" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>pca_australia</t>
+          <t>msfitnessaustralia</t>
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>11495</v>
+        <v>15579</v>
       </c>
       <c r="C18" s="27" t="n">
-        <v>11410</v>
+        <v>15466</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>85</v>
+        <v>113</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.0074</v>
+        <v>0.0073</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>icn.indonesia</t>
+          <t>nabbaaustralia</t>
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>1845</v>
+        <v>15804</v>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1843</v>
+        <v>15721</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>2</v>
+        <v>83</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0011</v>
+        <v>0.0053</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>nabbaaustralia</t>
+          <t>msfitnessaustralia_perth</t>
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>15807</v>
+        <v>1443</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>15793</v>
+        <v>1442</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0009</v>
+        <v>0.0007000000000000001</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H20" s="26" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_perth</t>
+          <t>icn.indonesia</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>1443</v>
+        <v>1838</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1444</v>
+        <v>1838</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E21" s="30" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>0</v>
+      </c>
+      <c r="E21" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H21" s="26" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
@@ -3497,24 +3501,24 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>2270</v>
+        <v>2276</v>
       </c>
       <c r="C22" s="27" t="n">
-        <v>2276</v>
+        <v>2277</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0026</v>
+        <v>-0.0004</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H22" s="26" t="n">
         <v>17</v>
@@ -3527,10 +3531,10 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>4590</v>
+        <v>4581</v>
       </c>
       <c r="C23" s="27" t="n">
-        <v>4629</v>
+        <v>4620</v>
       </c>
       <c r="D23" s="28" t="n">
         <v>-39</v>
@@ -3540,11 +3544,11 @@
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H23" s="26" t="n">
         <v>15</v>
@@ -3606,7 +3610,7 @@
       </c>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3617,14 +3621,14 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3409</v>
+        <v>3440</v>
       </c>
       <c r="C3" s="28" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3635,14 +3639,14 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6895</v>
+        <v>6927</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3653,14 +3657,14 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>7004</v>
+        <v>7042</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3671,14 +3675,14 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>3024</v>
+        <v>3060</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3689,14 +3693,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3625</v>
+        <v>3652</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3707,14 +3711,14 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4491</v>
+        <v>4510</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3725,14 +3729,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2892</v>
+        <v>2898</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3743,14 +3747,14 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4454</v>
+        <v>4460</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3761,14 +3765,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2792</v>
+        <v>2815</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>23</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3782,11 +3786,11 @@
         <v>922</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3797,14 +3801,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3231</v>
+        <v>3251</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>101</v>
+        <v>20</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3815,14 +3819,14 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1168</v>
+        <v>1173</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3833,14 +3837,14 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>1950</v>
+        <v>1955</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3853,10 +3857,12 @@
       <c r="B16" s="27" t="n">
         <v>814</v>
       </c>
-      <c r="C16" s="28" t="n"/>
+      <c r="C16" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3867,14 +3873,14 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>363</v>
+        <v>396</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3885,12 +3891,14 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>2125</v>
-      </c>
-      <c r="C18" s="28" t="n"/>
+        <v>2127</v>
+      </c>
+      <c r="C18" s="28" t="n">
+        <v>2</v>
+      </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3908,7 +3916,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3926,7 +3934,7 @@
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3937,14 +3945,14 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C21" s="28" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3970,7 @@
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3973,14 +3981,14 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="C23" s="28" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4037,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4059,7 +4067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D453"/>
+  <dimension ref="A1:D475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13130,6 +13138,446 @@
         </is>
       </c>
     </row>
+    <row r="454" ht="21" customHeight="1">
+      <c r="A454" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B454" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C454" s="27" t="n">
+        <v>9846</v>
+      </c>
+      <c r="D454" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="455" ht="21" customHeight="1">
+      <c r="A455" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B455" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C455" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="D455" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="456" ht="21" customHeight="1">
+      <c r="A456" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B456" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C456" s="27" t="n">
+        <v>1852</v>
+      </c>
+      <c r="D456" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="457" ht="21" customHeight="1">
+      <c r="A457" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B457" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C457" s="27" t="n">
+        <v>1838</v>
+      </c>
+      <c r="D457" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="458" ht="21" customHeight="1">
+      <c r="A458" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B458" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C458" s="27" t="n">
+        <v>4702</v>
+      </c>
+      <c r="D458" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="459" ht="21" customHeight="1">
+      <c r="A459" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B459" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C459" s="27" t="n">
+        <v>16320</v>
+      </c>
+      <c r="D459" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="460" ht="21" customHeight="1">
+      <c r="A460" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B460" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C460" s="27" t="n">
+        <v>1487</v>
+      </c>
+      <c r="D460" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="461" ht="21" customHeight="1">
+      <c r="A461" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B461" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C461" s="27" t="n">
+        <v>6903</v>
+      </c>
+      <c r="D461" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="462" ht="21" customHeight="1">
+      <c r="A462" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B462" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C462" s="27" t="n">
+        <v>2276</v>
+      </c>
+      <c r="D462" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="463" ht="21" customHeight="1">
+      <c r="A463" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B463" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C463" s="27" t="n">
+        <v>13226</v>
+      </c>
+      <c r="D463" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="464" ht="21" customHeight="1">
+      <c r="A464" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B464" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C464" s="27" t="n">
+        <v>11184</v>
+      </c>
+      <c r="D464" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="465" ht="21" customHeight="1">
+      <c r="A465" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B465" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C465" s="27" t="n">
+        <v>6610</v>
+      </c>
+      <c r="D465" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="466" ht="21" customHeight="1">
+      <c r="A466" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B466" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C466" s="27" t="n">
+        <v>18063</v>
+      </c>
+      <c r="D466" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="467" ht="21" customHeight="1">
+      <c r="A467" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B467" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C467" s="27" t="n">
+        <v>58222</v>
+      </c>
+      <c r="D467" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="468" ht="21" customHeight="1">
+      <c r="A468" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B468" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C468" s="27" t="n">
+        <v>15579</v>
+      </c>
+      <c r="D468" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="469" ht="21" customHeight="1">
+      <c r="A469" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B469" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C469" s="27" t="n">
+        <v>1443</v>
+      </c>
+      <c r="D469" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="470" ht="21" customHeight="1">
+      <c r="A470" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B470" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C470" s="27" t="n">
+        <v>974</v>
+      </c>
+      <c r="D470" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="471" ht="21" customHeight="1">
+      <c r="A471" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B471" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C471" s="27" t="n">
+        <v>15804</v>
+      </c>
+      <c r="D471" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="472" ht="21" customHeight="1">
+      <c r="A472" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B472" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C472" s="27" t="n">
+        <v>18778</v>
+      </c>
+      <c r="D472" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="473" ht="21" customHeight="1">
+      <c r="A473" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B473" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C473" s="27" t="n">
+        <v>11519</v>
+      </c>
+      <c r="D473" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="474" ht="21" customHeight="1">
+      <c r="A474" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B474" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C474" s="27" t="n">
+        <v>7505</v>
+      </c>
+      <c r="D474" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="475" ht="21" customHeight="1">
+      <c r="A475" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B475" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C475" s="27" t="n">
+        <v>4581</v>
+      </c>
+      <c r="D475" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-10-18
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 12 October 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 18 October 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,778</t>
+          <t>18,829</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+1.92%</t>
+          <t>+1.62%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+353 followers • 36 days</t>
+          <t>+300 followers • 35 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>58222</v>
+        <v>58175</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -1272,14 +1272,14 @@
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>430</v>
+        <v>608</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.1937</v>
+        <v>0.2697</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18778</v>
+        <v>18829</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
@@ -1306,14 +1306,14 @@
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.0417</v>
+        <v>0.0317</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,25 +1329,25 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>18063</v>
+        <v>18074</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@icn_act</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>55</v>
+        <v>135</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.0384</v>
+        <v>0.0294</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,25 +1363,25 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>16320</v>
+        <v>16314</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>@wnbfaustralia</t>
+          <t>@icn_sa</t>
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>253</v>
+        <v>183</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0349</v>
+        <v>0.0272</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,25 +1397,25 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15804</v>
+        <v>15767</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>@icn_sa</t>
+          <t>@wnbfaustralia</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.0278</v>
+        <v>0.0248</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>36d</t>
+          <t>35d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>58222</v>
+        <v>58175</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.1937</v>
+        <v>0.2697</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,7 +1826,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18778</v>
+        <v>18829</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.0417</v>
+        <v>0.0317</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,15 +1844,15 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>18063</v>
+        <v>18074</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@icn_act</t>
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.0384</v>
+        <v>0.0294</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,15 +1862,15 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16320</v>
+        <v>16314</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>@wnbfaustralia</t>
+          <t>@icn_sa</t>
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0349</v>
+        <v>0.0272</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,15 +1880,15 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15804</v>
+        <v>15767</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>@icn_sa</t>
+          <t>@wnbfaustralia</t>
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.0278</v>
+        <v>0.0248</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,21 +2002,21 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>58222</v>
+        <v>58175</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>683</v>
+        <v>291</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0119</v>
+        <v>0.005</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H2" s="27" t="n">
         <v>8186</v>
@@ -2040,27 +2040,27 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18778</v>
+        <v>18829</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>353</v>
+        <v>300</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0192</v>
+        <v>0.0162</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3440</v>
+        <v>3459</v>
       </c>
       <c r="I3" s="28" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
@@ -2078,27 +2078,27 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>18063</v>
+        <v>18074</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>228</v>
+        <v>209</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0128</v>
+        <v>0.0117</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6927</v>
+        <v>6941</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2116,27 +2116,27 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>16320</v>
+        <v>16314</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>284</v>
+        <v>179</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0177</v>
+        <v>0.0111</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>7042</v>
+        <v>7064</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
@@ -2154,27 +2154,27 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15804</v>
+        <v>15767</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0053</v>
+        <v>0.0033</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>3060</v>
+        <v>3074</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
@@ -2192,27 +2192,27 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15579</v>
+        <v>15581</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0073</v>
+        <v>0.0048</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3652</v>
+        <v>3675</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="J7" s="26" t="inlineStr">
         <is>
@@ -2230,27 +2230,27 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>13226</v>
+        <v>13227</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>333</v>
+        <v>264</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0258</v>
+        <v>0.0204</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4510</v>
+        <v>4512</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
@@ -2268,27 +2268,27 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11519</v>
+        <v>11562</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.0124</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2898</v>
+        <v>2913</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,27 +2306,27 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>11184</v>
+        <v>11173</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>187</v>
+        <v>155</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.017</v>
+        <v>0.0141</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H10" s="27" t="n">
-        <v>4460</v>
+        <v>4464</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
@@ -2344,27 +2344,27 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9846</v>
+        <v>9882</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>112</v>
+        <v>138</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0115</v>
+        <v>0.0142</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2815</v>
+        <v>2830</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
@@ -2382,21 +2382,21 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7505</v>
+        <v>7522</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>253</v>
+        <v>182</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0349</v>
+        <v>0.0248</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H12" s="27" t="n">
         <v>922</v>
@@ -2420,27 +2420,27 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6903</v>
+        <v>6913</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0278</v>
+        <v>0.0272</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3251</v>
+        <v>3270</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,27 +2458,27 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6610</v>
+        <v>6644</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0143</v>
+        <v>0.0161</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>1209</v>
+      </c>
+      <c r="I14" s="28" t="n">
         <v>36</v>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>1173</v>
-      </c>
-      <c r="I14" s="28" t="n">
-        <v>5</v>
       </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
@@ -2496,27 +2496,27 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4702</v>
+        <v>4734</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0242</v>
+        <v>0.0294</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H15" s="27" t="n">
-        <v>1955</v>
+        <v>1957</v>
       </c>
       <c r="I15" s="28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J15" s="26" t="inlineStr">
         <is>
@@ -2534,21 +2534,21 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4581</v>
+        <v>4573</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-39</v>
+        <v>-40</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H16" s="27" t="n">
         <v>814</v>
@@ -2572,27 +2572,27 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2650</v>
+        <v>2862</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>430</v>
+        <v>608</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.1937</v>
+        <v>0.2697</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>396</v>
+        <v>484</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -2613,24 +2613,24 @@
         <v>2276</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E18" s="30" t="n">
-        <v>-0.0004</v>
+        <v>0</v>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H18" s="27" t="n">
         <v>2127</v>
       </c>
       <c r="I18" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J18" s="26" t="inlineStr">
         <is>
@@ -2651,18 +2651,18 @@
         <v>1852</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.008199999999999999</v>
+        <v>0.0076</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H19" s="27" t="n">
         <v>208</v>
@@ -2686,21 +2686,21 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1838</v>
+        <v>1831</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="29" t="n">
-        <v>0</v>
+        <v>-10</v>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>-0.0054</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H20" s="27" t="n">
         <v>176</v>
@@ -2724,27 +2724,27 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1487</v>
+        <v>1489</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0.0384</v>
+        <v>0.0178</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>344</v>
+        <v>353</v>
       </c>
       <c r="I21" s="28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J21" s="26" t="inlineStr">
         <is>
@@ -2762,21 +2762,21 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1443</v>
+        <v>1441</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="29" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.0014</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H22" s="27" t="n">
         <v>1357</v>
@@ -2800,27 +2800,27 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>974</v>
+        <v>977</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.0417</v>
+        <v>0.0317</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>737</v>
+        <v>756</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
@@ -2901,24 +2901,24 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>2650</v>
+        <v>2862</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>2220</v>
+        <v>2254</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>430</v>
+        <v>608</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.1937</v>
+        <v>0.2697</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H2" s="26" t="n">
         <v>16</v>
@@ -2931,24 +2931,24 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>974</v>
+        <v>977</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>935</v>
+        <v>947</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0417</v>
+        <v>0.0317</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H3" s="26" t="n">
         <v>22</v>
@@ -2957,91 +2957,91 @@
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>icn_act</t>
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>1487</v>
+        <v>4734</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>1432</v>
+        <v>4599</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>55</v>
+        <v>135</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0384</v>
+        <v>0.0294</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H4" s="26" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" ht="21" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>wnbfaustralia</t>
+          <t>icn_sa</t>
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>7505</v>
+        <v>6913</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>7252</v>
+        <v>6730</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>253</v>
+        <v>183</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0349</v>
+        <v>0.0272</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>icn_sa</t>
+          <t>wnbfaustralia</t>
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>6903</v>
+        <v>7522</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>6716</v>
+        <v>7340</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0278</v>
+        <v>0.0248</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
@@ -3051,24 +3051,24 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>13226</v>
+        <v>13227</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>12893</v>
+        <v>12963</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>333</v>
+        <v>264</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0258</v>
+        <v>0.0204</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H7" s="26" t="n">
         <v>7</v>
@@ -3077,31 +3077,31 @@
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>icn_act</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4702</v>
+        <v>1489</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>4591</v>
+        <v>1463</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>111</v>
+        <v>26</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0242</v>
+        <v>0.0178</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
@@ -3111,24 +3111,24 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>18778</v>
+        <v>18829</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>18425</v>
+        <v>18529</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>353</v>
+        <v>300</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0192</v>
+        <v>0.0162</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H9" s="26" t="n">
         <v>2</v>
@@ -3137,241 +3137,241 @@
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>icn_nsw</t>
+          <t>icnnewzealand</t>
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>16320</v>
+        <v>6644</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>16036</v>
+        <v>6539</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>284</v>
+        <v>105</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0177</v>
+        <v>0.0161</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>icn_wa</t>
+          <t>anb.australia</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>11184</v>
+        <v>9882</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>10997</v>
+        <v>9744</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>187</v>
+        <v>138</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.017</v>
+        <v>0.0142</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>icnnewzealand</t>
+          <t>icn_wa</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>6610</v>
+        <v>11173</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>6517</v>
+        <v>11018</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>93</v>
+        <v>155</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0143</v>
+        <v>0.0141</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>icnqld</t>
+          <t>pca_australia</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>18063</v>
+        <v>11562</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>17835</v>
+        <v>11420</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>228</v>
+        <v>142</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0128</v>
+        <v>0.0124</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>icnqld</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>58222</v>
+        <v>18074</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>57539</v>
+        <v>17865</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>683</v>
+        <v>209</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0119</v>
+        <v>0.0117</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>anb.australia</t>
+          <t>icn_nsw</t>
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>9846</v>
+        <v>16314</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>9734</v>
+        <v>16135</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>112</v>
+        <v>179</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0115</v>
+        <v>0.0111</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H15" s="26" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>pca_australia</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>11519</v>
+        <v>1852</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>11413</v>
+        <v>1838</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>106</v>
+        <v>14</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.0076</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H16" s="26" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>1852</v>
+        <v>58175</v>
       </c>
       <c r="C17" s="27" t="n">
-        <v>1837</v>
+        <v>57884</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>15</v>
+        <v>291</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.008199999999999999</v>
+        <v>0.005</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H17" s="26" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
@@ -3381,24 +3381,24 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>15579</v>
+        <v>15581</v>
       </c>
       <c r="C18" s="27" t="n">
-        <v>15466</v>
+        <v>15507</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.0073</v>
+        <v>0.0048</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H18" s="26" t="n">
         <v>6</v>
@@ -3411,24 +3411,24 @@
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>15804</v>
+        <v>15767</v>
       </c>
       <c r="C19" s="27" t="n">
-        <v>15721</v>
+        <v>15715</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0053</v>
+        <v>0.0033</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H19" s="26" t="n">
         <v>5</v>
@@ -3441,24 +3441,24 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>1443</v>
+        <v>1441</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1442</v>
+        <v>1439</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.0014</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H20" s="26" t="n">
         <v>21</v>
@@ -3467,14 +3467,14 @@
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>icn.indonesia</t>
+          <t>icn_tasmania</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>1838</v>
+        <v>2276</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1838</v>
+        <v>2276</v>
       </c>
       <c r="D21" s="28" t="n">
         <v>0</v>
@@ -3484,44 +3484,44 @@
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H21" s="26" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>icn_tasmania</t>
+          <t>icn.indonesia</t>
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>2276</v>
+        <v>1831</v>
       </c>
       <c r="C22" s="27" t="n">
-        <v>2277</v>
+        <v>1841</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-1</v>
+        <v>-10</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0004</v>
+        <v>-0.0054</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H22" s="26" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" ht="21" customHeight="1">
@@ -3531,24 +3531,24 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>4581</v>
+        <v>4573</v>
       </c>
       <c r="C23" s="27" t="n">
-        <v>4620</v>
+        <v>4613</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-39</v>
+        <v>-40</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H23" s="26" t="n">
         <v>15</v>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3621,14 +3621,14 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3440</v>
+        <v>3459</v>
       </c>
       <c r="C3" s="28" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3639,14 +3639,14 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6927</v>
+        <v>6941</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3657,14 +3657,14 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>7042</v>
+        <v>7064</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3675,14 +3675,14 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>3060</v>
+        <v>3074</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3693,14 +3693,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3652</v>
+        <v>3675</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3711,14 +3711,14 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4510</v>
+        <v>4512</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3729,14 +3729,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2898</v>
+        <v>2913</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3747,14 +3747,14 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4460</v>
+        <v>4464</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3765,14 +3765,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2815</v>
+        <v>2830</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3790,7 +3790,7 @@
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3801,14 +3801,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3251</v>
+        <v>3270</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3819,14 +3819,14 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1173</v>
+        <v>1209</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3837,14 +3837,14 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>1955</v>
+        <v>1957</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3873,14 +3873,14 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>396</v>
+        <v>484</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3894,11 +3894,11 @@
         <v>2127</v>
       </c>
       <c r="C18" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3945,14 +3945,14 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>344</v>
+        <v>353</v>
       </c>
       <c r="C21" s="28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3981,14 +3981,14 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>737</v>
+        <v>756</v>
       </c>
       <c r="C23" s="28" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D475"/>
+  <dimension ref="A1:D497"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13578,6 +13578,446 @@
         </is>
       </c>
     </row>
+    <row r="476" ht="21" customHeight="1">
+      <c r="A476" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B476" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C476" s="27" t="n">
+        <v>9882</v>
+      </c>
+      <c r="D476" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="477" ht="21" customHeight="1">
+      <c r="A477" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B477" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C477" s="27" t="n">
+        <v>2862</v>
+      </c>
+      <c r="D477" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="478" ht="21" customHeight="1">
+      <c r="A478" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B478" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C478" s="27" t="n">
+        <v>1852</v>
+      </c>
+      <c r="D478" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="479" ht="21" customHeight="1">
+      <c r="A479" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B479" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C479" s="27" t="n">
+        <v>1831</v>
+      </c>
+      <c r="D479" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="480" ht="21" customHeight="1">
+      <c r="A480" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B480" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C480" s="27" t="n">
+        <v>4734</v>
+      </c>
+      <c r="D480" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="481" ht="21" customHeight="1">
+      <c r="A481" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B481" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C481" s="27" t="n">
+        <v>16314</v>
+      </c>
+      <c r="D481" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="482" ht="21" customHeight="1">
+      <c r="A482" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B482" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C482" s="27" t="n">
+        <v>1489</v>
+      </c>
+      <c r="D482" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="483" ht="21" customHeight="1">
+      <c r="A483" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B483" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C483" s="27" t="n">
+        <v>6913</v>
+      </c>
+      <c r="D483" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="484" ht="21" customHeight="1">
+      <c r="A484" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B484" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C484" s="27" t="n">
+        <v>2276</v>
+      </c>
+      <c r="D484" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="485" ht="21" customHeight="1">
+      <c r="A485" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B485" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C485" s="27" t="n">
+        <v>13227</v>
+      </c>
+      <c r="D485" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="486" ht="21" customHeight="1">
+      <c r="A486" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B486" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C486" s="27" t="n">
+        <v>11173</v>
+      </c>
+      <c r="D486" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="487" ht="21" customHeight="1">
+      <c r="A487" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B487" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C487" s="27" t="n">
+        <v>6644</v>
+      </c>
+      <c r="D487" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="488" ht="21" customHeight="1">
+      <c r="A488" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B488" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C488" s="27" t="n">
+        <v>18074</v>
+      </c>
+      <c r="D488" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="489" ht="21" customHeight="1">
+      <c r="A489" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B489" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C489" s="27" t="n">
+        <v>58175</v>
+      </c>
+      <c r="D489" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="490" ht="21" customHeight="1">
+      <c r="A490" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B490" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C490" s="27" t="n">
+        <v>15581</v>
+      </c>
+      <c r="D490" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="491" ht="21" customHeight="1">
+      <c r="A491" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B491" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C491" s="27" t="n">
+        <v>1441</v>
+      </c>
+      <c r="D491" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="492" ht="21" customHeight="1">
+      <c r="A492" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B492" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C492" s="27" t="n">
+        <v>977</v>
+      </c>
+      <c r="D492" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="493" ht="21" customHeight="1">
+      <c r="A493" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B493" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C493" s="27" t="n">
+        <v>15767</v>
+      </c>
+      <c r="D493" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="494" ht="21" customHeight="1">
+      <c r="A494" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B494" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C494" s="27" t="n">
+        <v>18829</v>
+      </c>
+      <c r="D494" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="495" ht="21" customHeight="1">
+      <c r="A495" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B495" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C495" s="27" t="n">
+        <v>11562</v>
+      </c>
+      <c r="D495" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="496" ht="21" customHeight="1">
+      <c r="A496" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B496" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C496" s="27" t="n">
+        <v>7522</v>
+      </c>
+      <c r="D496" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="497" ht="21" customHeight="1">
+      <c r="A497" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B497" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C497" s="27" t="n">
+        <v>4573</v>
+      </c>
+      <c r="D497" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-10-25
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -106,13 +106,13 @@
     <font>
       <name val="Aptos"/>
       <b val="1"/>
-      <color rgb="0012B76A"/>
+      <color rgb="00F04438"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Aptos"/>
       <b val="1"/>
-      <color rgb="00F04438"/>
+      <color rgb="0012B76A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 18 October 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 25 October 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,829</t>
+          <t>18,864</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+1.62%</t>
+          <t>+1.41%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+300 followers • 35 days</t>
+          <t>+263 followers • 35 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>58175</v>
+        <v>58162</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -1272,10 +1272,10 @@
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>608</v>
+        <v>600</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.2697</v>
+        <v>0.2626</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18829</v>
+        <v>18864</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
@@ -1306,10 +1306,10 @@
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.0317</v>
+        <v>0.0357</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>18074</v>
+        <v>18107</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
@@ -1340,10 +1340,10 @@
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.0294</v>
+        <v>0.0271</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>16314</v>
+        <v>16315</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
@@ -1374,10 +1374,10 @@
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0272</v>
+        <v>0.0269</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
@@ -1397,21 +1397,21 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15767</v>
+        <v>15690</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>@wnbfaustralia</t>
+          <t>@pca_australia</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.0248</v>
+        <v>0.0179</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>58175</v>
+        <v>58162</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.2697</v>
+        <v>0.2626</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,7 +1826,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18829</v>
+        <v>18864</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.0317</v>
+        <v>0.0357</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>18074</v>
+        <v>18107</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.0294</v>
+        <v>0.0271</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16314</v>
+        <v>16315</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0272</v>
+        <v>0.0269</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,15 +1880,15 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15767</v>
+        <v>15690</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>@wnbfaustralia</t>
+          <t>@pca_australia</t>
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.0248</v>
+        <v>0.0179</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,28 +2002,24 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>58175</v>
+        <v>58162</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>291</v>
+        <v>-72</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.005</v>
+        <v>-0.0012</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H2" s="27" t="n">
-        <v>8186</v>
-      </c>
-      <c r="I2" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="H2" s="27" t="n"/>
+      <c r="I2" s="28" t="n"/>
       <c r="J2" s="26" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2040,28 +2036,24 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18829</v>
+        <v>18864</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>300</v>
-      </c>
-      <c r="E3" s="29" t="n">
-        <v>0.0162</v>
+        <v>263</v>
+      </c>
+      <c r="E3" s="30" t="n">
+        <v>0.0141</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H3" s="27" t="n">
-        <v>3459</v>
-      </c>
-      <c r="I3" s="28" t="n">
-        <v>19</v>
-      </c>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="28" t="n"/>
       <c r="J3" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2078,28 +2070,24 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>18074</v>
+        <v>18107</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>209</v>
-      </c>
-      <c r="E4" s="29" t="n">
-        <v>0.0117</v>
+        <v>199</v>
+      </c>
+      <c r="E4" s="30" t="n">
+        <v>0.0111</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H4" s="27" t="n">
-        <v>6941</v>
-      </c>
-      <c r="I4" s="28" t="n">
-        <v>14</v>
-      </c>
+      <c r="H4" s="27" t="n"/>
+      <c r="I4" s="28" t="n"/>
       <c r="J4" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2116,28 +2104,24 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>16314</v>
+        <v>16315</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>179</v>
-      </c>
-      <c r="E5" s="29" t="n">
-        <v>0.0111</v>
+        <v>98</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <v>0.006</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H5" s="27" t="n">
-        <v>7064</v>
-      </c>
-      <c r="I5" s="28" t="n">
-        <v>22</v>
-      </c>
+      <c r="H5" s="27" t="n"/>
+      <c r="I5" s="28" t="n"/>
       <c r="J5" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2154,28 +2138,24 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15767</v>
+        <v>15690</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>52</v>
+        <v>-30</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0033</v>
+        <v>-0.0019</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H6" s="27" t="n">
-        <v>3074</v>
-      </c>
-      <c r="I6" s="28" t="n">
-        <v>14</v>
-      </c>
+      <c r="H6" s="27" t="n"/>
+      <c r="I6" s="28" t="n"/>
       <c r="J6" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2192,27 +2172,27 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15581</v>
+        <v>15579</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>74</v>
-      </c>
-      <c r="E7" s="29" t="n">
-        <v>0.0048</v>
+        <v>45</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>0.0029</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3675</v>
+        <v>3685</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="J7" s="26" t="inlineStr">
         <is>
@@ -2230,27 +2210,27 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>13227</v>
+        <v>13231</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>264</v>
-      </c>
-      <c r="E8" s="29" t="n">
-        <v>0.0204</v>
+        <v>212</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <v>0.0163</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4512</v>
+        <v>4515</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
@@ -2268,27 +2248,27 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11562</v>
+        <v>11642</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>142</v>
-      </c>
-      <c r="E9" s="29" t="n">
-        <v>0.0124</v>
+        <v>205</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <v>0.0179</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2913</v>
+        <v>3005</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>15</v>
+        <v>92</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,28 +2286,24 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>11173</v>
+        <v>11185</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>155</v>
-      </c>
-      <c r="E10" s="29" t="n">
-        <v>0.0141</v>
+        <v>97</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>0.008699999999999999</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H10" s="27" t="n">
-        <v>4464</v>
-      </c>
-      <c r="I10" s="28" t="n">
-        <v>4</v>
-      </c>
+      <c r="H10" s="27" t="n"/>
+      <c r="I10" s="28" t="n"/>
       <c r="J10" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2344,27 +2320,27 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9882</v>
+        <v>9924</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>138</v>
-      </c>
-      <c r="E11" s="29" t="n">
-        <v>0.0142</v>
+        <v>165</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>0.0169</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2830</v>
+        <v>2859</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
@@ -2382,27 +2358,27 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7522</v>
+        <v>7526</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>182</v>
-      </c>
-      <c r="E12" s="29" t="n">
-        <v>0.0248</v>
+        <v>93</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>0.0125</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
@@ -2420,27 +2396,27 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6913</v>
+        <v>6918</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>183</v>
-      </c>
-      <c r="E13" s="29" t="n">
-        <v>0.0272</v>
+        <v>181</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>0.0269</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3270</v>
+        <v>3272</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,27 +2434,27 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6644</v>
+        <v>6654</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>105</v>
-      </c>
-      <c r="E14" s="29" t="n">
-        <v>0.0161</v>
+        <v>94</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>0.0143</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1209</v>
+        <v>1222</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
@@ -2496,27 +2472,27 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4734</v>
+        <v>4740</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>135</v>
-      </c>
-      <c r="E15" s="29" t="n">
-        <v>0.0294</v>
+        <v>125</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>0.0271</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H15" s="27" t="n">
-        <v>1957</v>
+        <v>1960</v>
       </c>
       <c r="I15" s="28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J15" s="26" t="inlineStr">
         <is>
@@ -2534,28 +2510,24 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4573</v>
+        <v>4561</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-40</v>
-      </c>
-      <c r="E16" s="30" t="n">
-        <v>-0.008699999999999999</v>
+        <v>-45</v>
+      </c>
+      <c r="E16" s="29" t="n">
+        <v>-0.0098</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H16" s="27" t="n">
-        <v>814</v>
-      </c>
-      <c r="I16" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="H16" s="27" t="n"/>
+      <c r="I16" s="28" t="n"/>
       <c r="J16" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2572,28 +2544,24 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2862</v>
+        <v>2885</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>608</v>
-      </c>
-      <c r="E17" s="29" t="n">
-        <v>0.2697</v>
+        <v>600</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>0.2626</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H17" s="27" t="n">
-        <v>484</v>
-      </c>
-      <c r="I17" s="28" t="n">
-        <v>88</v>
-      </c>
+      <c r="H17" s="27" t="n"/>
+      <c r="I17" s="28" t="n"/>
       <c r="J17" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2613,25 +2581,21 @@
         <v>2276</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="29" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>0.0013</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H18" s="27" t="n">
-        <v>2127</v>
-      </c>
-      <c r="I18" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="H18" s="27" t="n"/>
+      <c r="I18" s="28" t="n"/>
       <c r="J18" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2648,28 +2612,24 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1852</v>
+        <v>1848</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>14</v>
-      </c>
-      <c r="E19" s="29" t="n">
-        <v>0.0076</v>
+        <v>7</v>
+      </c>
+      <c r="E19" s="30" t="n">
+        <v>0.0038</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H19" s="27" t="n">
-        <v>208</v>
-      </c>
-      <c r="I19" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="H19" s="27" t="n"/>
+      <c r="I19" s="28" t="n"/>
       <c r="J19" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2686,28 +2646,24 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1831</v>
+        <v>1835</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>-10</v>
-      </c>
-      <c r="E20" s="30" t="n">
-        <v>-0.0054</v>
+        <v>-9</v>
+      </c>
+      <c r="E20" s="29" t="n">
+        <v>-0.0049</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H20" s="27" t="n">
-        <v>176</v>
-      </c>
-      <c r="I20" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="H20" s="27" t="n"/>
+      <c r="I20" s="28" t="n"/>
       <c r="J20" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2724,27 +2680,27 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1489</v>
+        <v>1486</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="E21" s="29" t="n">
-        <v>0.0178</v>
+        <v>11</v>
+      </c>
+      <c r="E21" s="30" t="n">
+        <v>0.0075</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="I21" s="28" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J21" s="26" t="inlineStr">
         <is>
@@ -2762,28 +2718,24 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1441</v>
+        <v>1439</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="E22" s="29" t="n">
-        <v>0.0014</v>
+        <v>-0.0021</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H22" s="27" t="n">
-        <v>1357</v>
-      </c>
-      <c r="I22" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="H22" s="27" t="n"/>
+      <c r="I22" s="28" t="n"/>
       <c r="J22" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2800,28 +2752,24 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>977</v>
+        <v>986</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>30</v>
-      </c>
-      <c r="E23" s="29" t="n">
-        <v>0.0317</v>
+        <v>34</v>
+      </c>
+      <c r="E23" s="30" t="n">
+        <v>0.0357</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H23" s="27" t="n">
-        <v>756</v>
-      </c>
-      <c r="I23" s="28" t="n">
-        <v>19</v>
-      </c>
+      <c r="H23" s="27" t="n"/>
+      <c r="I23" s="28" t="n"/>
       <c r="J23" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2901,20 +2849,20 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>2862</v>
+        <v>2885</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>2254</v>
+        <v>2285</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>608</v>
-      </c>
-      <c r="E2" s="29" t="n">
-        <v>0.2697</v>
+        <v>600</v>
+      </c>
+      <c r="E2" s="30" t="n">
+        <v>0.2626</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G2" s="26" t="n">
@@ -2931,20 +2879,20 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>977</v>
+        <v>986</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>947</v>
+        <v>952</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>30</v>
-      </c>
-      <c r="E3" s="29" t="n">
-        <v>0.0317</v>
+        <v>34</v>
+      </c>
+      <c r="E3" s="30" t="n">
+        <v>0.0357</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G3" s="26" t="n">
@@ -2961,20 +2909,20 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>4734</v>
+        <v>4740</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>4599</v>
+        <v>4615</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>135</v>
-      </c>
-      <c r="E4" s="29" t="n">
-        <v>0.0294</v>
+        <v>125</v>
+      </c>
+      <c r="E4" s="30" t="n">
+        <v>0.0271</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G4" s="26" t="n">
@@ -2991,20 +2939,20 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6913</v>
+        <v>6918</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>6730</v>
+        <v>6737</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>183</v>
-      </c>
-      <c r="E5" s="29" t="n">
-        <v>0.0272</v>
+        <v>181</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <v>0.0269</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G5" s="26" t="n">
@@ -3017,271 +2965,271 @@
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>wnbfaustralia</t>
+          <t>pca_australia</t>
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>7522</v>
+        <v>11642</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>7340</v>
+        <v>11437</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>182</v>
-      </c>
-      <c r="E6" s="29" t="n">
-        <v>0.0248</v>
+        <v>205</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <v>0.0179</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>icn_victoria</t>
+          <t>anb.australia</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>13227</v>
+        <v>9924</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>12963</v>
+        <v>9759</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>264</v>
-      </c>
-      <c r="E7" s="29" t="n">
-        <v>0.0204</v>
+        <v>165</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>0.0169</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G7" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>icn_victoria</t>
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>1489</v>
+        <v>13231</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>1463</v>
+        <v>13019</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="E8" s="29" t="n">
-        <v>0.0178</v>
+        <v>212</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <v>0.0163</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G8" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>nbaaustralia_official</t>
+          <t>icnnewzealand</t>
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>18829</v>
+        <v>6654</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>18529</v>
+        <v>6560</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>300</v>
-      </c>
-      <c r="E9" s="29" t="n">
-        <v>0.0162</v>
+        <v>94</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <v>0.0143</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G9" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>icnnewzealand</t>
+          <t>nbaaustralia_official</t>
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>6644</v>
+        <v>18864</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>6539</v>
+        <v>18601</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>105</v>
-      </c>
-      <c r="E10" s="29" t="n">
-        <v>0.0161</v>
+        <v>263</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>0.0141</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G10" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>anb.australia</t>
+          <t>wnbfaustralia</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>9882</v>
+        <v>7526</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9744</v>
+        <v>7433</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>138</v>
-      </c>
-      <c r="E11" s="29" t="n">
-        <v>0.0142</v>
+        <v>93</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>0.0125</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G11" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>icn_wa</t>
+          <t>icnqld</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>11173</v>
+        <v>18107</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>11018</v>
+        <v>17908</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>155</v>
-      </c>
-      <c r="E12" s="29" t="n">
-        <v>0.0141</v>
+        <v>199</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>0.0111</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>pca_australia</t>
+          <t>icn_wa</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>11562</v>
+        <v>11185</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>11420</v>
+        <v>11088</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>142</v>
-      </c>
-      <c r="E13" s="29" t="n">
-        <v>0.0124</v>
+        <v>97</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>0.008699999999999999</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G13" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>icnqld</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>18074</v>
+        <v>1486</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>17865</v>
+        <v>1475</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>209</v>
-      </c>
-      <c r="E14" s="29" t="n">
-        <v>0.0117</v>
+        <v>11</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>0.0075</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
@@ -3291,20 +3239,20 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>16314</v>
+        <v>16315</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>16135</v>
+        <v>16217</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>179</v>
-      </c>
-      <c r="E15" s="29" t="n">
-        <v>0.0111</v>
+        <v>98</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>0.006</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
@@ -3321,20 +3269,20 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>1852</v>
+        <v>1848</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>1838</v>
+        <v>1841</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>14</v>
-      </c>
-      <c r="E16" s="29" t="n">
-        <v>0.0076</v>
+        <v>7</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>0.0038</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
@@ -3347,151 +3295,151 @@
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>msfitnessaustralia</t>
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>58175</v>
+        <v>15579</v>
       </c>
       <c r="C17" s="27" t="n">
-        <v>57884</v>
+        <v>15534</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>291</v>
-      </c>
-      <c r="E17" s="29" t="n">
-        <v>0.005</v>
+        <v>45</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>0.0029</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H17" s="26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia</t>
+          <t>icn_tasmania</t>
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>15581</v>
+        <v>2276</v>
       </c>
       <c r="C18" s="27" t="n">
-        <v>15507</v>
+        <v>2273</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>74</v>
-      </c>
-      <c r="E18" s="29" t="n">
-        <v>0.0048</v>
+        <v>3</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>0.0013</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>nabbaaustralia</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>15767</v>
+        <v>58162</v>
       </c>
       <c r="C19" s="27" t="n">
-        <v>15715</v>
+        <v>58234</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>52</v>
+        <v>-72</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0033</v>
+        <v>-0.0012</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_perth</t>
+          <t>nabbaaustralia</t>
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>1441</v>
+        <v>15690</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1439</v>
+        <v>15720</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>2</v>
+        <v>-30</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0014</v>
+        <v>-0.0019</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G20" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H20" s="26" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>icn_tasmania</t>
+          <t>msfitnessaustralia_perth</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>2276</v>
+        <v>1439</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>2276</v>
+        <v>1442</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0</v>
+        <v>-0.0021</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G21" s="26" t="n">
         <v>35</v>
       </c>
       <c r="H21" s="26" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
@@ -3501,20 +3449,20 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>1831</v>
+        <v>1835</v>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1841</v>
+        <v>1844</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-10</v>
-      </c>
-      <c r="E22" s="30" t="n">
-        <v>-0.0054</v>
+        <v>-9</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>-0.0049</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G22" s="26" t="n">
@@ -3531,20 +3479,20 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>4573</v>
+        <v>4561</v>
       </c>
       <c r="C23" s="27" t="n">
-        <v>4613</v>
+        <v>4606</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-40</v>
-      </c>
-      <c r="E23" s="30" t="n">
-        <v>-0.008699999999999999</v>
+        <v>-45</v>
+      </c>
+      <c r="E23" s="29" t="n">
+        <v>-0.0098</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G23" s="26" t="n">
@@ -3602,15 +3550,11 @@
           <t>ifbbproleagueoz</t>
         </is>
       </c>
-      <c r="B2" s="27" t="n">
-        <v>8186</v>
-      </c>
-      <c r="C2" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="B2" s="27" t="n"/>
+      <c r="C2" s="28" t="n"/>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3620,15 +3564,11 @@
           <t>nbaaustralia_official</t>
         </is>
       </c>
-      <c r="B3" s="27" t="n">
-        <v>3459</v>
-      </c>
-      <c r="C3" s="28" t="n">
-        <v>19</v>
-      </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="28" t="n"/>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3638,15 +3578,11 @@
           <t>icnqld</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n">
-        <v>6941</v>
-      </c>
-      <c r="C4" s="28" t="n">
-        <v>14</v>
-      </c>
+      <c r="B4" s="27" t="n"/>
+      <c r="C4" s="28" t="n"/>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3656,15 +3592,11 @@
           <t>icn_nsw</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n">
-        <v>7064</v>
-      </c>
-      <c r="C5" s="28" t="n">
-        <v>22</v>
-      </c>
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="28" t="n"/>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3674,15 +3606,11 @@
           <t>nabbaaustralia</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
-        <v>3074</v>
-      </c>
-      <c r="C6" s="28" t="n">
-        <v>14</v>
-      </c>
+      <c r="B6" s="27" t="n"/>
+      <c r="C6" s="28" t="n"/>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3693,14 +3621,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3675</v>
+        <v>3685</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3711,14 +3639,14 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4512</v>
+        <v>4515</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3729,14 +3657,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2913</v>
+        <v>3005</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>15</v>
+        <v>92</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3746,15 +3674,11 @@
           <t>icn_wa</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
-        <v>4464</v>
-      </c>
-      <c r="C10" s="28" t="n">
-        <v>4</v>
-      </c>
+      <c r="B10" s="27" t="n"/>
+      <c r="C10" s="28" t="n"/>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3765,14 +3689,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2830</v>
+        <v>2859</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3783,14 +3707,14 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3801,14 +3725,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3270</v>
+        <v>3272</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3819,14 +3743,14 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1209</v>
+        <v>1222</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3837,14 +3761,14 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>1957</v>
+        <v>1960</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3854,15 +3778,11 @@
           <t>ynf_australia</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
-        <v>814</v>
-      </c>
-      <c r="C16" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="B16" s="27" t="n"/>
+      <c r="C16" s="28" t="n"/>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3872,15 +3792,11 @@
           <t>cbrfitexpo</t>
         </is>
       </c>
-      <c r="B17" s="27" t="n">
-        <v>484</v>
-      </c>
-      <c r="C17" s="28" t="n">
-        <v>88</v>
-      </c>
+      <c r="B17" s="27" t="n"/>
+      <c r="C17" s="28" t="n"/>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3890,15 +3806,11 @@
           <t>icn_tasmania</t>
         </is>
       </c>
-      <c r="B18" s="27" t="n">
-        <v>2127</v>
-      </c>
-      <c r="C18" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="B18" s="27" t="n"/>
+      <c r="C18" s="28" t="n"/>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3908,15 +3820,11 @@
           <t>dfba_global</t>
         </is>
       </c>
-      <c r="B19" s="27" t="n">
-        <v>208</v>
-      </c>
-      <c r="C19" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="B19" s="27" t="n"/>
+      <c r="C19" s="28" t="n"/>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3926,15 +3834,11 @@
           <t>icn.indonesia</t>
         </is>
       </c>
-      <c r="B20" s="27" t="n">
-        <v>176</v>
-      </c>
-      <c r="C20" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="B20" s="27" t="n"/>
+      <c r="C20" s="28" t="n"/>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3945,14 +3849,14 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C21" s="28" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3962,15 +3866,11 @@
           <t>msfitnessaustralia_perth</t>
         </is>
       </c>
-      <c r="B22" s="27" t="n">
-        <v>1357</v>
-      </c>
-      <c r="C22" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="B22" s="27" t="n"/>
+      <c r="C22" s="28" t="n"/>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3980,15 +3880,11 @@
           <t>msfitnessaustralia_vic</t>
         </is>
       </c>
-      <c r="B23" s="27" t="n">
-        <v>756</v>
-      </c>
-      <c r="C23" s="28" t="n">
-        <v>19</v>
-      </c>
+      <c r="B23" s="27" t="n"/>
+      <c r="C23" s="28" t="n"/>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4037,7 +3933,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4067,7 +3963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D497"/>
+  <dimension ref="A1:D519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -14018,6 +13914,446 @@
         </is>
       </c>
     </row>
+    <row r="498" ht="21" customHeight="1">
+      <c r="A498" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B498" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C498" s="27" t="n">
+        <v>9924</v>
+      </c>
+      <c r="D498" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="499" ht="21" customHeight="1">
+      <c r="A499" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B499" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C499" s="27" t="n">
+        <v>2885</v>
+      </c>
+      <c r="D499" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="500" ht="21" customHeight="1">
+      <c r="A500" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B500" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C500" s="27" t="n">
+        <v>1848</v>
+      </c>
+      <c r="D500" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="501" ht="21" customHeight="1">
+      <c r="A501" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B501" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C501" s="27" t="n">
+        <v>1835</v>
+      </c>
+      <c r="D501" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="502" ht="21" customHeight="1">
+      <c r="A502" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B502" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C502" s="27" t="n">
+        <v>4740</v>
+      </c>
+      <c r="D502" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="503" ht="21" customHeight="1">
+      <c r="A503" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B503" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C503" s="27" t="n">
+        <v>16315</v>
+      </c>
+      <c r="D503" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="504" ht="21" customHeight="1">
+      <c r="A504" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B504" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C504" s="27" t="n">
+        <v>1486</v>
+      </c>
+      <c r="D504" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="505" ht="21" customHeight="1">
+      <c r="A505" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B505" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C505" s="27" t="n">
+        <v>6918</v>
+      </c>
+      <c r="D505" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="506" ht="21" customHeight="1">
+      <c r="A506" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B506" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C506" s="27" t="n">
+        <v>2276</v>
+      </c>
+      <c r="D506" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="507" ht="21" customHeight="1">
+      <c r="A507" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B507" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C507" s="27" t="n">
+        <v>13231</v>
+      </c>
+      <c r="D507" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="508" ht="21" customHeight="1">
+      <c r="A508" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B508" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C508" s="27" t="n">
+        <v>11185</v>
+      </c>
+      <c r="D508" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="509" ht="21" customHeight="1">
+      <c r="A509" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B509" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C509" s="27" t="n">
+        <v>6654</v>
+      </c>
+      <c r="D509" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="510" ht="21" customHeight="1">
+      <c r="A510" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B510" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C510" s="27" t="n">
+        <v>18107</v>
+      </c>
+      <c r="D510" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="511" ht="21" customHeight="1">
+      <c r="A511" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B511" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C511" s="27" t="n">
+        <v>58162</v>
+      </c>
+      <c r="D511" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="512" ht="21" customHeight="1">
+      <c r="A512" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B512" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C512" s="27" t="n">
+        <v>15579</v>
+      </c>
+      <c r="D512" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="513" ht="21" customHeight="1">
+      <c r="A513" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B513" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C513" s="27" t="n">
+        <v>1439</v>
+      </c>
+      <c r="D513" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="514" ht="21" customHeight="1">
+      <c r="A514" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B514" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C514" s="27" t="n">
+        <v>986</v>
+      </c>
+      <c r="D514" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="515" ht="21" customHeight="1">
+      <c r="A515" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B515" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C515" s="27" t="n">
+        <v>15690</v>
+      </c>
+      <c r="D515" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="516" ht="21" customHeight="1">
+      <c r="A516" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B516" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C516" s="27" t="n">
+        <v>18864</v>
+      </c>
+      <c r="D516" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="517" ht="21" customHeight="1">
+      <c r="A517" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B517" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C517" s="27" t="n">
+        <v>11642</v>
+      </c>
+      <c r="D517" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="518" ht="21" customHeight="1">
+      <c r="A518" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B518" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C518" s="27" t="n">
+        <v>7526</v>
+      </c>
+      <c r="D518" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="519" ht="21" customHeight="1">
+      <c r="A519" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B519" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C519" s="27" t="n">
+        <v>4561</v>
+      </c>
+      <c r="D519" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>